<commit_message>
Aba Provisionado: economia = provisionado − gasto
Nova aba Provisionado (por implantação ou por categoria de custo).
Economia passa a ser provisionado − gasto nas implantações concluídas;
em andamento mostram o saldo disponível. Gráficos viram provisionado × gasto
por implantação e por categoria, com o estouro em vermelho.
Planilha-modelo e README atualizados.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013DBwNxsZwLrtk7qvNchaRT
</commit_message>
<xml_diff>
--- a/modelo/planilha-implantacoes.xlsx
+++ b/modelo/planilha-implantacoes.xlsx
@@ -10,8 +10,9 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Como usar" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Clientes" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Implantacoes" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lancamentos" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Economias" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Provisionado" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lancamentos" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Economias" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -444,7 +445,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A12"/>
+  <dimension ref="A1:A15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="120" customWidth="1" min="1" max="1"/>
@@ -463,7 +464,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>O painel lê 4 abas. Não renomeie as abas nem os cabeçalhos da linha 1.</t>
+          <t>O painel lê 5 abas. Não renomeie as abas nem os cabeçalhos da linha 1.</t>
         </is>
       </c>
     </row>
@@ -477,50 +478,71 @@
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Implantacoes — uma linha por implantação. id_cliente vem da aba Clientes. valor_orcado = orçamento aprovado.</t>
+          <t>Implantacoes — uma linha por implantação. id_cliente vem da aba Clientes.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Lancamentos — cada custo da implantação (nota, folha, empreiteiro, deslocamento).</t>
+          <t>Provisionado — quanto você PODIA gastar em cada implantação. Pode ser uma linha só (categoria em branco)</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">     Deixe data_pagamento em branco enquanto não pagar: o painel marca 'A vencer' ou 'Vencido' pelo vencimento.</t>
+          <t xml:space="preserve">     ou uma linha por categoria de custo, para ver onde sobrou ou estourou.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Economias — só negociação na compra e reaproveitamento de estoque.</t>
+          <t>Lancamentos — cada custo da implantação (nota, folha, empreiteiro, deslocamento).</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">     'Execução abaixo do orçado' é calculada sozinha: orçado − custo − (negociação + estoque), só nas concluídas.</t>
+          <t xml:space="preserve">     Deixe data_pagamento em branco enquanto não pagar: o painel marca 'A vencer' ou 'Vencido' pelo vencimento.</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="2" t="inlineStr"/>
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>Economia = provisionado − gasto, contada quando a implantação fica Concluída. Antes disso o painel mostra o saldo disponível.</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>Status da implantação: Planejada, Em andamento ou Concluída.</t>
+          <t>Economias — opcional: registre negociação na compra e reaproveitamento de estoque para ver de onde veio a economia.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">     O resto (economia − negociação − estoque) aparece como execução.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>Status da implantação: Planejada, Em andamento ou Concluída.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
         <is>
           <t>As linhas atuais são exemplo — apague e lance as implantações reais.</t>
         </is>
@@ -692,7 +714,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H500"/>
+  <dimension ref="A1:G500"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -702,7 +724,6 @@
     <col width="14" customWidth="1" min="5" max="5"/>
     <col width="16" customWidth="1" min="6" max="6"/>
     <col width="15" customWidth="1" min="7" max="7"/>
-    <col width="16" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -741,11 +762,6 @@
           <t>status</t>
         </is>
       </c>
-      <c r="H1" s="3" t="inlineStr">
-        <is>
-          <t>valor_orcado</t>
-        </is>
-      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -779,9 +795,6 @@
           <t>Concluída</t>
         </is>
       </c>
-      <c r="H2" s="5" t="n">
-        <v>48000</v>
-      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -815,9 +828,6 @@
           <t>Concluída</t>
         </is>
       </c>
-      <c r="H3" s="5" t="n">
-        <v>31500</v>
-      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -851,9 +861,6 @@
           <t>Concluída</t>
         </is>
       </c>
-      <c r="H4" s="5" t="n">
-        <v>22800</v>
-      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -887,9 +894,6 @@
           <t>Concluída</t>
         </is>
       </c>
-      <c r="H5" s="5" t="n">
-        <v>27400</v>
-      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -923,9 +927,6 @@
           <t>Concluída</t>
         </is>
       </c>
-      <c r="H6" s="5" t="n">
-        <v>16900</v>
-      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -959,9 +960,6 @@
           <t>Concluída</t>
         </is>
       </c>
-      <c r="H7" s="5" t="n">
-        <v>52300</v>
-      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -993,9 +991,6 @@
           <t>Em andamento</t>
         </is>
       </c>
-      <c r="H8" s="5" t="n">
-        <v>35600</v>
-      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1027,9 +1022,6 @@
           <t>Em andamento</t>
         </is>
       </c>
-      <c r="H9" s="5" t="n">
-        <v>19800</v>
-      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1061,9 +1053,6 @@
           <t>Em andamento</t>
         </is>
       </c>
-      <c r="H10" s="5" t="n">
-        <v>41200</v>
-      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1094,2455 +1083,1963 @@
         <is>
           <t>Planejada</t>
         </is>
-      </c>
-      <c r="H11" s="5" t="n">
-        <v>18600</v>
       </c>
     </row>
     <row r="12">
       <c r="E12" s="4" t="n"/>
       <c r="F12" s="4" t="n"/>
-      <c r="H12" s="5" t="n"/>
     </row>
     <row r="13">
       <c r="E13" s="4" t="n"/>
       <c r="F13" s="4" t="n"/>
-      <c r="H13" s="5" t="n"/>
     </row>
     <row r="14">
       <c r="E14" s="4" t="n"/>
       <c r="F14" s="4" t="n"/>
-      <c r="H14" s="5" t="n"/>
     </row>
     <row r="15">
       <c r="E15" s="4" t="n"/>
       <c r="F15" s="4" t="n"/>
-      <c r="H15" s="5" t="n"/>
     </row>
     <row r="16">
       <c r="E16" s="4" t="n"/>
       <c r="F16" s="4" t="n"/>
-      <c r="H16" s="5" t="n"/>
     </row>
     <row r="17">
       <c r="E17" s="4" t="n"/>
       <c r="F17" s="4" t="n"/>
-      <c r="H17" s="5" t="n"/>
     </row>
     <row r="18">
       <c r="E18" s="4" t="n"/>
       <c r="F18" s="4" t="n"/>
-      <c r="H18" s="5" t="n"/>
     </row>
     <row r="19">
       <c r="E19" s="4" t="n"/>
       <c r="F19" s="4" t="n"/>
-      <c r="H19" s="5" t="n"/>
     </row>
     <row r="20">
       <c r="E20" s="4" t="n"/>
       <c r="F20" s="4" t="n"/>
-      <c r="H20" s="5" t="n"/>
     </row>
     <row r="21">
       <c r="E21" s="4" t="n"/>
       <c r="F21" s="4" t="n"/>
-      <c r="H21" s="5" t="n"/>
     </row>
     <row r="22">
       <c r="E22" s="4" t="n"/>
       <c r="F22" s="4" t="n"/>
-      <c r="H22" s="5" t="n"/>
     </row>
     <row r="23">
       <c r="E23" s="4" t="n"/>
       <c r="F23" s="4" t="n"/>
-      <c r="H23" s="5" t="n"/>
     </row>
     <row r="24">
       <c r="E24" s="4" t="n"/>
       <c r="F24" s="4" t="n"/>
-      <c r="H24" s="5" t="n"/>
     </row>
     <row r="25">
       <c r="E25" s="4" t="n"/>
       <c r="F25" s="4" t="n"/>
-      <c r="H25" s="5" t="n"/>
     </row>
     <row r="26">
       <c r="E26" s="4" t="n"/>
       <c r="F26" s="4" t="n"/>
-      <c r="H26" s="5" t="n"/>
     </row>
     <row r="27">
       <c r="E27" s="4" t="n"/>
       <c r="F27" s="4" t="n"/>
-      <c r="H27" s="5" t="n"/>
     </row>
     <row r="28">
       <c r="E28" s="4" t="n"/>
       <c r="F28" s="4" t="n"/>
-      <c r="H28" s="5" t="n"/>
     </row>
     <row r="29">
       <c r="E29" s="4" t="n"/>
       <c r="F29" s="4" t="n"/>
-      <c r="H29" s="5" t="n"/>
     </row>
     <row r="30">
       <c r="E30" s="4" t="n"/>
       <c r="F30" s="4" t="n"/>
-      <c r="H30" s="5" t="n"/>
     </row>
     <row r="31">
       <c r="E31" s="4" t="n"/>
       <c r="F31" s="4" t="n"/>
-      <c r="H31" s="5" t="n"/>
     </row>
     <row r="32">
       <c r="E32" s="4" t="n"/>
       <c r="F32" s="4" t="n"/>
-      <c r="H32" s="5" t="n"/>
     </row>
     <row r="33">
       <c r="E33" s="4" t="n"/>
       <c r="F33" s="4" t="n"/>
-      <c r="H33" s="5" t="n"/>
     </row>
     <row r="34">
       <c r="E34" s="4" t="n"/>
       <c r="F34" s="4" t="n"/>
-      <c r="H34" s="5" t="n"/>
     </row>
     <row r="35">
       <c r="E35" s="4" t="n"/>
       <c r="F35" s="4" t="n"/>
-      <c r="H35" s="5" t="n"/>
     </row>
     <row r="36">
       <c r="E36" s="4" t="n"/>
       <c r="F36" s="4" t="n"/>
-      <c r="H36" s="5" t="n"/>
     </row>
     <row r="37">
       <c r="E37" s="4" t="n"/>
       <c r="F37" s="4" t="n"/>
-      <c r="H37" s="5" t="n"/>
     </row>
     <row r="38">
       <c r="E38" s="4" t="n"/>
       <c r="F38" s="4" t="n"/>
-      <c r="H38" s="5" t="n"/>
     </row>
     <row r="39">
       <c r="E39" s="4" t="n"/>
       <c r="F39" s="4" t="n"/>
-      <c r="H39" s="5" t="n"/>
     </row>
     <row r="40">
       <c r="E40" s="4" t="n"/>
       <c r="F40" s="4" t="n"/>
-      <c r="H40" s="5" t="n"/>
     </row>
     <row r="41">
       <c r="E41" s="4" t="n"/>
       <c r="F41" s="4" t="n"/>
-      <c r="H41" s="5" t="n"/>
     </row>
     <row r="42">
       <c r="E42" s="4" t="n"/>
       <c r="F42" s="4" t="n"/>
-      <c r="H42" s="5" t="n"/>
     </row>
     <row r="43">
       <c r="E43" s="4" t="n"/>
       <c r="F43" s="4" t="n"/>
-      <c r="H43" s="5" t="n"/>
     </row>
     <row r="44">
       <c r="E44" s="4" t="n"/>
       <c r="F44" s="4" t="n"/>
-      <c r="H44" s="5" t="n"/>
     </row>
     <row r="45">
       <c r="E45" s="4" t="n"/>
       <c r="F45" s="4" t="n"/>
-      <c r="H45" s="5" t="n"/>
     </row>
     <row r="46">
       <c r="E46" s="4" t="n"/>
       <c r="F46" s="4" t="n"/>
-      <c r="H46" s="5" t="n"/>
     </row>
     <row r="47">
       <c r="E47" s="4" t="n"/>
       <c r="F47" s="4" t="n"/>
-      <c r="H47" s="5" t="n"/>
     </row>
     <row r="48">
       <c r="E48" s="4" t="n"/>
       <c r="F48" s="4" t="n"/>
-      <c r="H48" s="5" t="n"/>
     </row>
     <row r="49">
       <c r="E49" s="4" t="n"/>
       <c r="F49" s="4" t="n"/>
-      <c r="H49" s="5" t="n"/>
     </row>
     <row r="50">
       <c r="E50" s="4" t="n"/>
       <c r="F50" s="4" t="n"/>
-      <c r="H50" s="5" t="n"/>
     </row>
     <row r="51">
       <c r="E51" s="4" t="n"/>
       <c r="F51" s="4" t="n"/>
-      <c r="H51" s="5" t="n"/>
     </row>
     <row r="52">
       <c r="E52" s="4" t="n"/>
       <c r="F52" s="4" t="n"/>
-      <c r="H52" s="5" t="n"/>
     </row>
     <row r="53">
       <c r="E53" s="4" t="n"/>
       <c r="F53" s="4" t="n"/>
-      <c r="H53" s="5" t="n"/>
     </row>
     <row r="54">
       <c r="E54" s="4" t="n"/>
       <c r="F54" s="4" t="n"/>
-      <c r="H54" s="5" t="n"/>
     </row>
     <row r="55">
       <c r="E55" s="4" t="n"/>
       <c r="F55" s="4" t="n"/>
-      <c r="H55" s="5" t="n"/>
     </row>
     <row r="56">
       <c r="E56" s="4" t="n"/>
       <c r="F56" s="4" t="n"/>
-      <c r="H56" s="5" t="n"/>
     </row>
     <row r="57">
       <c r="E57" s="4" t="n"/>
       <c r="F57" s="4" t="n"/>
-      <c r="H57" s="5" t="n"/>
     </row>
     <row r="58">
       <c r="E58" s="4" t="n"/>
       <c r="F58" s="4" t="n"/>
-      <c r="H58" s="5" t="n"/>
     </row>
     <row r="59">
       <c r="E59" s="4" t="n"/>
       <c r="F59" s="4" t="n"/>
-      <c r="H59" s="5" t="n"/>
     </row>
     <row r="60">
       <c r="E60" s="4" t="n"/>
       <c r="F60" s="4" t="n"/>
-      <c r="H60" s="5" t="n"/>
     </row>
     <row r="61">
       <c r="E61" s="4" t="n"/>
       <c r="F61" s="4" t="n"/>
-      <c r="H61" s="5" t="n"/>
     </row>
     <row r="62">
       <c r="E62" s="4" t="n"/>
       <c r="F62" s="4" t="n"/>
-      <c r="H62" s="5" t="n"/>
     </row>
     <row r="63">
       <c r="E63" s="4" t="n"/>
       <c r="F63" s="4" t="n"/>
-      <c r="H63" s="5" t="n"/>
     </row>
     <row r="64">
       <c r="E64" s="4" t="n"/>
       <c r="F64" s="4" t="n"/>
-      <c r="H64" s="5" t="n"/>
     </row>
     <row r="65">
       <c r="E65" s="4" t="n"/>
       <c r="F65" s="4" t="n"/>
-      <c r="H65" s="5" t="n"/>
     </row>
     <row r="66">
       <c r="E66" s="4" t="n"/>
       <c r="F66" s="4" t="n"/>
-      <c r="H66" s="5" t="n"/>
     </row>
     <row r="67">
       <c r="E67" s="4" t="n"/>
       <c r="F67" s="4" t="n"/>
-      <c r="H67" s="5" t="n"/>
     </row>
     <row r="68">
       <c r="E68" s="4" t="n"/>
       <c r="F68" s="4" t="n"/>
-      <c r="H68" s="5" t="n"/>
     </row>
     <row r="69">
       <c r="E69" s="4" t="n"/>
       <c r="F69" s="4" t="n"/>
-      <c r="H69" s="5" t="n"/>
     </row>
     <row r="70">
       <c r="E70" s="4" t="n"/>
       <c r="F70" s="4" t="n"/>
-      <c r="H70" s="5" t="n"/>
     </row>
     <row r="71">
       <c r="E71" s="4" t="n"/>
       <c r="F71" s="4" t="n"/>
-      <c r="H71" s="5" t="n"/>
     </row>
     <row r="72">
       <c r="E72" s="4" t="n"/>
       <c r="F72" s="4" t="n"/>
-      <c r="H72" s="5" t="n"/>
     </row>
     <row r="73">
       <c r="E73" s="4" t="n"/>
       <c r="F73" s="4" t="n"/>
-      <c r="H73" s="5" t="n"/>
     </row>
     <row r="74">
       <c r="E74" s="4" t="n"/>
       <c r="F74" s="4" t="n"/>
-      <c r="H74" s="5" t="n"/>
     </row>
     <row r="75">
       <c r="E75" s="4" t="n"/>
       <c r="F75" s="4" t="n"/>
-      <c r="H75" s="5" t="n"/>
     </row>
     <row r="76">
       <c r="E76" s="4" t="n"/>
       <c r="F76" s="4" t="n"/>
-      <c r="H76" s="5" t="n"/>
     </row>
     <row r="77">
       <c r="E77" s="4" t="n"/>
       <c r="F77" s="4" t="n"/>
-      <c r="H77" s="5" t="n"/>
     </row>
     <row r="78">
       <c r="E78" s="4" t="n"/>
       <c r="F78" s="4" t="n"/>
-      <c r="H78" s="5" t="n"/>
     </row>
     <row r="79">
       <c r="E79" s="4" t="n"/>
       <c r="F79" s="4" t="n"/>
-      <c r="H79" s="5" t="n"/>
     </row>
     <row r="80">
       <c r="E80" s="4" t="n"/>
       <c r="F80" s="4" t="n"/>
-      <c r="H80" s="5" t="n"/>
     </row>
     <row r="81">
       <c r="E81" s="4" t="n"/>
       <c r="F81" s="4" t="n"/>
-      <c r="H81" s="5" t="n"/>
     </row>
     <row r="82">
       <c r="E82" s="4" t="n"/>
       <c r="F82" s="4" t="n"/>
-      <c r="H82" s="5" t="n"/>
     </row>
     <row r="83">
       <c r="E83" s="4" t="n"/>
       <c r="F83" s="4" t="n"/>
-      <c r="H83" s="5" t="n"/>
     </row>
     <row r="84">
       <c r="E84" s="4" t="n"/>
       <c r="F84" s="4" t="n"/>
-      <c r="H84" s="5" t="n"/>
     </row>
     <row r="85">
       <c r="E85" s="4" t="n"/>
       <c r="F85" s="4" t="n"/>
-      <c r="H85" s="5" t="n"/>
     </row>
     <row r="86">
       <c r="E86" s="4" t="n"/>
       <c r="F86" s="4" t="n"/>
-      <c r="H86" s="5" t="n"/>
     </row>
     <row r="87">
       <c r="E87" s="4" t="n"/>
       <c r="F87" s="4" t="n"/>
-      <c r="H87" s="5" t="n"/>
     </row>
     <row r="88">
       <c r="E88" s="4" t="n"/>
       <c r="F88" s="4" t="n"/>
-      <c r="H88" s="5" t="n"/>
     </row>
     <row r="89">
       <c r="E89" s="4" t="n"/>
       <c r="F89" s="4" t="n"/>
-      <c r="H89" s="5" t="n"/>
     </row>
     <row r="90">
       <c r="E90" s="4" t="n"/>
       <c r="F90" s="4" t="n"/>
-      <c r="H90" s="5" t="n"/>
     </row>
     <row r="91">
       <c r="E91" s="4" t="n"/>
       <c r="F91" s="4" t="n"/>
-      <c r="H91" s="5" t="n"/>
     </row>
     <row r="92">
       <c r="E92" s="4" t="n"/>
       <c r="F92" s="4" t="n"/>
-      <c r="H92" s="5" t="n"/>
     </row>
     <row r="93">
       <c r="E93" s="4" t="n"/>
       <c r="F93" s="4" t="n"/>
-      <c r="H93" s="5" t="n"/>
     </row>
     <row r="94">
       <c r="E94" s="4" t="n"/>
       <c r="F94" s="4" t="n"/>
-      <c r="H94" s="5" t="n"/>
     </row>
     <row r="95">
       <c r="E95" s="4" t="n"/>
       <c r="F95" s="4" t="n"/>
-      <c r="H95" s="5" t="n"/>
     </row>
     <row r="96">
       <c r="E96" s="4" t="n"/>
       <c r="F96" s="4" t="n"/>
-      <c r="H96" s="5" t="n"/>
     </row>
     <row r="97">
       <c r="E97" s="4" t="n"/>
       <c r="F97" s="4" t="n"/>
-      <c r="H97" s="5" t="n"/>
     </row>
     <row r="98">
       <c r="E98" s="4" t="n"/>
       <c r="F98" s="4" t="n"/>
-      <c r="H98" s="5" t="n"/>
     </row>
     <row r="99">
       <c r="E99" s="4" t="n"/>
       <c r="F99" s="4" t="n"/>
-      <c r="H99" s="5" t="n"/>
     </row>
     <row r="100">
       <c r="E100" s="4" t="n"/>
       <c r="F100" s="4" t="n"/>
-      <c r="H100" s="5" t="n"/>
     </row>
     <row r="101">
       <c r="E101" s="4" t="n"/>
       <c r="F101" s="4" t="n"/>
-      <c r="H101" s="5" t="n"/>
     </row>
     <row r="102">
       <c r="E102" s="4" t="n"/>
       <c r="F102" s="4" t="n"/>
-      <c r="H102" s="5" t="n"/>
     </row>
     <row r="103">
       <c r="E103" s="4" t="n"/>
       <c r="F103" s="4" t="n"/>
-      <c r="H103" s="5" t="n"/>
     </row>
     <row r="104">
       <c r="E104" s="4" t="n"/>
       <c r="F104" s="4" t="n"/>
-      <c r="H104" s="5" t="n"/>
     </row>
     <row r="105">
       <c r="E105" s="4" t="n"/>
       <c r="F105" s="4" t="n"/>
-      <c r="H105" s="5" t="n"/>
     </row>
     <row r="106">
       <c r="E106" s="4" t="n"/>
       <c r="F106" s="4" t="n"/>
-      <c r="H106" s="5" t="n"/>
     </row>
     <row r="107">
       <c r="E107" s="4" t="n"/>
       <c r="F107" s="4" t="n"/>
-      <c r="H107" s="5" t="n"/>
     </row>
     <row r="108">
       <c r="E108" s="4" t="n"/>
       <c r="F108" s="4" t="n"/>
-      <c r="H108" s="5" t="n"/>
     </row>
     <row r="109">
       <c r="E109" s="4" t="n"/>
       <c r="F109" s="4" t="n"/>
-      <c r="H109" s="5" t="n"/>
     </row>
     <row r="110">
       <c r="E110" s="4" t="n"/>
       <c r="F110" s="4" t="n"/>
-      <c r="H110" s="5" t="n"/>
     </row>
     <row r="111">
       <c r="E111" s="4" t="n"/>
       <c r="F111" s="4" t="n"/>
-      <c r="H111" s="5" t="n"/>
     </row>
     <row r="112">
       <c r="E112" s="4" t="n"/>
       <c r="F112" s="4" t="n"/>
-      <c r="H112" s="5" t="n"/>
     </row>
     <row r="113">
       <c r="E113" s="4" t="n"/>
       <c r="F113" s="4" t="n"/>
-      <c r="H113" s="5" t="n"/>
     </row>
     <row r="114">
       <c r="E114" s="4" t="n"/>
       <c r="F114" s="4" t="n"/>
-      <c r="H114" s="5" t="n"/>
     </row>
     <row r="115">
       <c r="E115" s="4" t="n"/>
       <c r="F115" s="4" t="n"/>
-      <c r="H115" s="5" t="n"/>
     </row>
     <row r="116">
       <c r="E116" s="4" t="n"/>
       <c r="F116" s="4" t="n"/>
-      <c r="H116" s="5" t="n"/>
     </row>
     <row r="117">
       <c r="E117" s="4" t="n"/>
       <c r="F117" s="4" t="n"/>
-      <c r="H117" s="5" t="n"/>
     </row>
     <row r="118">
       <c r="E118" s="4" t="n"/>
       <c r="F118" s="4" t="n"/>
-      <c r="H118" s="5" t="n"/>
     </row>
     <row r="119">
       <c r="E119" s="4" t="n"/>
       <c r="F119" s="4" t="n"/>
-      <c r="H119" s="5" t="n"/>
     </row>
     <row r="120">
       <c r="E120" s="4" t="n"/>
       <c r="F120" s="4" t="n"/>
-      <c r="H120" s="5" t="n"/>
     </row>
     <row r="121">
       <c r="E121" s="4" t="n"/>
       <c r="F121" s="4" t="n"/>
-      <c r="H121" s="5" t="n"/>
     </row>
     <row r="122">
       <c r="E122" s="4" t="n"/>
       <c r="F122" s="4" t="n"/>
-      <c r="H122" s="5" t="n"/>
     </row>
     <row r="123">
       <c r="E123" s="4" t="n"/>
       <c r="F123" s="4" t="n"/>
-      <c r="H123" s="5" t="n"/>
     </row>
     <row r="124">
       <c r="E124" s="4" t="n"/>
       <c r="F124" s="4" t="n"/>
-      <c r="H124" s="5" t="n"/>
     </row>
     <row r="125">
       <c r="E125" s="4" t="n"/>
       <c r="F125" s="4" t="n"/>
-      <c r="H125" s="5" t="n"/>
     </row>
     <row r="126">
       <c r="E126" s="4" t="n"/>
       <c r="F126" s="4" t="n"/>
-      <c r="H126" s="5" t="n"/>
     </row>
     <row r="127">
       <c r="E127" s="4" t="n"/>
       <c r="F127" s="4" t="n"/>
-      <c r="H127" s="5" t="n"/>
     </row>
     <row r="128">
       <c r="E128" s="4" t="n"/>
       <c r="F128" s="4" t="n"/>
-      <c r="H128" s="5" t="n"/>
     </row>
     <row r="129">
       <c r="E129" s="4" t="n"/>
       <c r="F129" s="4" t="n"/>
-      <c r="H129" s="5" t="n"/>
     </row>
     <row r="130">
       <c r="E130" s="4" t="n"/>
       <c r="F130" s="4" t="n"/>
-      <c r="H130" s="5" t="n"/>
     </row>
     <row r="131">
       <c r="E131" s="4" t="n"/>
       <c r="F131" s="4" t="n"/>
-      <c r="H131" s="5" t="n"/>
     </row>
     <row r="132">
       <c r="E132" s="4" t="n"/>
       <c r="F132" s="4" t="n"/>
-      <c r="H132" s="5" t="n"/>
     </row>
     <row r="133">
       <c r="E133" s="4" t="n"/>
       <c r="F133" s="4" t="n"/>
-      <c r="H133" s="5" t="n"/>
     </row>
     <row r="134">
       <c r="E134" s="4" t="n"/>
       <c r="F134" s="4" t="n"/>
-      <c r="H134" s="5" t="n"/>
     </row>
     <row r="135">
       <c r="E135" s="4" t="n"/>
       <c r="F135" s="4" t="n"/>
-      <c r="H135" s="5" t="n"/>
     </row>
     <row r="136">
       <c r="E136" s="4" t="n"/>
       <c r="F136" s="4" t="n"/>
-      <c r="H136" s="5" t="n"/>
     </row>
     <row r="137">
       <c r="E137" s="4" t="n"/>
       <c r="F137" s="4" t="n"/>
-      <c r="H137" s="5" t="n"/>
     </row>
     <row r="138">
       <c r="E138" s="4" t="n"/>
       <c r="F138" s="4" t="n"/>
-      <c r="H138" s="5" t="n"/>
     </row>
     <row r="139">
       <c r="E139" s="4" t="n"/>
       <c r="F139" s="4" t="n"/>
-      <c r="H139" s="5" t="n"/>
     </row>
     <row r="140">
       <c r="E140" s="4" t="n"/>
       <c r="F140" s="4" t="n"/>
-      <c r="H140" s="5" t="n"/>
     </row>
     <row r="141">
       <c r="E141" s="4" t="n"/>
       <c r="F141" s="4" t="n"/>
-      <c r="H141" s="5" t="n"/>
     </row>
     <row r="142">
       <c r="E142" s="4" t="n"/>
       <c r="F142" s="4" t="n"/>
-      <c r="H142" s="5" t="n"/>
     </row>
     <row r="143">
       <c r="E143" s="4" t="n"/>
       <c r="F143" s="4" t="n"/>
-      <c r="H143" s="5" t="n"/>
     </row>
     <row r="144">
       <c r="E144" s="4" t="n"/>
       <c r="F144" s="4" t="n"/>
-      <c r="H144" s="5" t="n"/>
     </row>
     <row r="145">
       <c r="E145" s="4" t="n"/>
       <c r="F145" s="4" t="n"/>
-      <c r="H145" s="5" t="n"/>
     </row>
     <row r="146">
       <c r="E146" s="4" t="n"/>
       <c r="F146" s="4" t="n"/>
-      <c r="H146" s="5" t="n"/>
     </row>
     <row r="147">
       <c r="E147" s="4" t="n"/>
       <c r="F147" s="4" t="n"/>
-      <c r="H147" s="5" t="n"/>
     </row>
     <row r="148">
       <c r="E148" s="4" t="n"/>
       <c r="F148" s="4" t="n"/>
-      <c r="H148" s="5" t="n"/>
     </row>
     <row r="149">
       <c r="E149" s="4" t="n"/>
       <c r="F149" s="4" t="n"/>
-      <c r="H149" s="5" t="n"/>
     </row>
     <row r="150">
       <c r="E150" s="4" t="n"/>
       <c r="F150" s="4" t="n"/>
-      <c r="H150" s="5" t="n"/>
     </row>
     <row r="151">
       <c r="E151" s="4" t="n"/>
       <c r="F151" s="4" t="n"/>
-      <c r="H151" s="5" t="n"/>
     </row>
     <row r="152">
       <c r="E152" s="4" t="n"/>
       <c r="F152" s="4" t="n"/>
-      <c r="H152" s="5" t="n"/>
     </row>
     <row r="153">
       <c r="E153" s="4" t="n"/>
       <c r="F153" s="4" t="n"/>
-      <c r="H153" s="5" t="n"/>
     </row>
     <row r="154">
       <c r="E154" s="4" t="n"/>
       <c r="F154" s="4" t="n"/>
-      <c r="H154" s="5" t="n"/>
     </row>
     <row r="155">
       <c r="E155" s="4" t="n"/>
       <c r="F155" s="4" t="n"/>
-      <c r="H155" s="5" t="n"/>
     </row>
     <row r="156">
       <c r="E156" s="4" t="n"/>
       <c r="F156" s="4" t="n"/>
-      <c r="H156" s="5" t="n"/>
     </row>
     <row r="157">
       <c r="E157" s="4" t="n"/>
       <c r="F157" s="4" t="n"/>
-      <c r="H157" s="5" t="n"/>
     </row>
     <row r="158">
       <c r="E158" s="4" t="n"/>
       <c r="F158" s="4" t="n"/>
-      <c r="H158" s="5" t="n"/>
     </row>
     <row r="159">
       <c r="E159" s="4" t="n"/>
       <c r="F159" s="4" t="n"/>
-      <c r="H159" s="5" t="n"/>
     </row>
     <row r="160">
       <c r="E160" s="4" t="n"/>
       <c r="F160" s="4" t="n"/>
-      <c r="H160" s="5" t="n"/>
     </row>
     <row r="161">
       <c r="E161" s="4" t="n"/>
       <c r="F161" s="4" t="n"/>
-      <c r="H161" s="5" t="n"/>
     </row>
     <row r="162">
       <c r="E162" s="4" t="n"/>
       <c r="F162" s="4" t="n"/>
-      <c r="H162" s="5" t="n"/>
     </row>
     <row r="163">
       <c r="E163" s="4" t="n"/>
       <c r="F163" s="4" t="n"/>
-      <c r="H163" s="5" t="n"/>
     </row>
     <row r="164">
       <c r="E164" s="4" t="n"/>
       <c r="F164" s="4" t="n"/>
-      <c r="H164" s="5" t="n"/>
     </row>
     <row r="165">
       <c r="E165" s="4" t="n"/>
       <c r="F165" s="4" t="n"/>
-      <c r="H165" s="5" t="n"/>
     </row>
     <row r="166">
       <c r="E166" s="4" t="n"/>
       <c r="F166" s="4" t="n"/>
-      <c r="H166" s="5" t="n"/>
     </row>
     <row r="167">
       <c r="E167" s="4" t="n"/>
       <c r="F167" s="4" t="n"/>
-      <c r="H167" s="5" t="n"/>
     </row>
     <row r="168">
       <c r="E168" s="4" t="n"/>
       <c r="F168" s="4" t="n"/>
-      <c r="H168" s="5" t="n"/>
     </row>
     <row r="169">
       <c r="E169" s="4" t="n"/>
       <c r="F169" s="4" t="n"/>
-      <c r="H169" s="5" t="n"/>
     </row>
     <row r="170">
       <c r="E170" s="4" t="n"/>
       <c r="F170" s="4" t="n"/>
-      <c r="H170" s="5" t="n"/>
     </row>
     <row r="171">
       <c r="E171" s="4" t="n"/>
       <c r="F171" s="4" t="n"/>
-      <c r="H171" s="5" t="n"/>
     </row>
     <row r="172">
       <c r="E172" s="4" t="n"/>
       <c r="F172" s="4" t="n"/>
-      <c r="H172" s="5" t="n"/>
     </row>
     <row r="173">
       <c r="E173" s="4" t="n"/>
       <c r="F173" s="4" t="n"/>
-      <c r="H173" s="5" t="n"/>
     </row>
     <row r="174">
       <c r="E174" s="4" t="n"/>
       <c r="F174" s="4" t="n"/>
-      <c r="H174" s="5" t="n"/>
     </row>
     <row r="175">
       <c r="E175" s="4" t="n"/>
       <c r="F175" s="4" t="n"/>
-      <c r="H175" s="5" t="n"/>
     </row>
     <row r="176">
       <c r="E176" s="4" t="n"/>
       <c r="F176" s="4" t="n"/>
-      <c r="H176" s="5" t="n"/>
     </row>
     <row r="177">
       <c r="E177" s="4" t="n"/>
       <c r="F177" s="4" t="n"/>
-      <c r="H177" s="5" t="n"/>
     </row>
     <row r="178">
       <c r="E178" s="4" t="n"/>
       <c r="F178" s="4" t="n"/>
-      <c r="H178" s="5" t="n"/>
     </row>
     <row r="179">
       <c r="E179" s="4" t="n"/>
       <c r="F179" s="4" t="n"/>
-      <c r="H179" s="5" t="n"/>
     </row>
     <row r="180">
       <c r="E180" s="4" t="n"/>
       <c r="F180" s="4" t="n"/>
-      <c r="H180" s="5" t="n"/>
     </row>
     <row r="181">
       <c r="E181" s="4" t="n"/>
       <c r="F181" s="4" t="n"/>
-      <c r="H181" s="5" t="n"/>
     </row>
     <row r="182">
       <c r="E182" s="4" t="n"/>
       <c r="F182" s="4" t="n"/>
-      <c r="H182" s="5" t="n"/>
     </row>
     <row r="183">
       <c r="E183" s="4" t="n"/>
       <c r="F183" s="4" t="n"/>
-      <c r="H183" s="5" t="n"/>
     </row>
     <row r="184">
       <c r="E184" s="4" t="n"/>
       <c r="F184" s="4" t="n"/>
-      <c r="H184" s="5" t="n"/>
     </row>
     <row r="185">
       <c r="E185" s="4" t="n"/>
       <c r="F185" s="4" t="n"/>
-      <c r="H185" s="5" t="n"/>
     </row>
     <row r="186">
       <c r="E186" s="4" t="n"/>
       <c r="F186" s="4" t="n"/>
-      <c r="H186" s="5" t="n"/>
     </row>
     <row r="187">
       <c r="E187" s="4" t="n"/>
       <c r="F187" s="4" t="n"/>
-      <c r="H187" s="5" t="n"/>
     </row>
     <row r="188">
       <c r="E188" s="4" t="n"/>
       <c r="F188" s="4" t="n"/>
-      <c r="H188" s="5" t="n"/>
     </row>
     <row r="189">
       <c r="E189" s="4" t="n"/>
       <c r="F189" s="4" t="n"/>
-      <c r="H189" s="5" t="n"/>
     </row>
     <row r="190">
       <c r="E190" s="4" t="n"/>
       <c r="F190" s="4" t="n"/>
-      <c r="H190" s="5" t="n"/>
     </row>
     <row r="191">
       <c r="E191" s="4" t="n"/>
       <c r="F191" s="4" t="n"/>
-      <c r="H191" s="5" t="n"/>
     </row>
     <row r="192">
       <c r="E192" s="4" t="n"/>
       <c r="F192" s="4" t="n"/>
-      <c r="H192" s="5" t="n"/>
     </row>
     <row r="193">
       <c r="E193" s="4" t="n"/>
       <c r="F193" s="4" t="n"/>
-      <c r="H193" s="5" t="n"/>
     </row>
     <row r="194">
       <c r="E194" s="4" t="n"/>
       <c r="F194" s="4" t="n"/>
-      <c r="H194" s="5" t="n"/>
     </row>
     <row r="195">
       <c r="E195" s="4" t="n"/>
       <c r="F195" s="4" t="n"/>
-      <c r="H195" s="5" t="n"/>
     </row>
     <row r="196">
       <c r="E196" s="4" t="n"/>
       <c r="F196" s="4" t="n"/>
-      <c r="H196" s="5" t="n"/>
     </row>
     <row r="197">
       <c r="E197" s="4" t="n"/>
       <c r="F197" s="4" t="n"/>
-      <c r="H197" s="5" t="n"/>
     </row>
     <row r="198">
       <c r="E198" s="4" t="n"/>
       <c r="F198" s="4" t="n"/>
-      <c r="H198" s="5" t="n"/>
     </row>
     <row r="199">
       <c r="E199" s="4" t="n"/>
       <c r="F199" s="4" t="n"/>
-      <c r="H199" s="5" t="n"/>
     </row>
     <row r="200">
       <c r="E200" s="4" t="n"/>
       <c r="F200" s="4" t="n"/>
-      <c r="H200" s="5" t="n"/>
     </row>
     <row r="201">
       <c r="E201" s="4" t="n"/>
       <c r="F201" s="4" t="n"/>
-      <c r="H201" s="5" t="n"/>
     </row>
     <row r="202">
       <c r="E202" s="4" t="n"/>
       <c r="F202" s="4" t="n"/>
-      <c r="H202" s="5" t="n"/>
     </row>
     <row r="203">
       <c r="E203" s="4" t="n"/>
       <c r="F203" s="4" t="n"/>
-      <c r="H203" s="5" t="n"/>
     </row>
     <row r="204">
       <c r="E204" s="4" t="n"/>
       <c r="F204" s="4" t="n"/>
-      <c r="H204" s="5" t="n"/>
     </row>
     <row r="205">
       <c r="E205" s="4" t="n"/>
       <c r="F205" s="4" t="n"/>
-      <c r="H205" s="5" t="n"/>
     </row>
     <row r="206">
       <c r="E206" s="4" t="n"/>
       <c r="F206" s="4" t="n"/>
-      <c r="H206" s="5" t="n"/>
     </row>
     <row r="207">
       <c r="E207" s="4" t="n"/>
       <c r="F207" s="4" t="n"/>
-      <c r="H207" s="5" t="n"/>
     </row>
     <row r="208">
       <c r="E208" s="4" t="n"/>
       <c r="F208" s="4" t="n"/>
-      <c r="H208" s="5" t="n"/>
     </row>
     <row r="209">
       <c r="E209" s="4" t="n"/>
       <c r="F209" s="4" t="n"/>
-      <c r="H209" s="5" t="n"/>
     </row>
     <row r="210">
       <c r="E210" s="4" t="n"/>
       <c r="F210" s="4" t="n"/>
-      <c r="H210" s="5" t="n"/>
     </row>
     <row r="211">
       <c r="E211" s="4" t="n"/>
       <c r="F211" s="4" t="n"/>
-      <c r="H211" s="5" t="n"/>
     </row>
     <row r="212">
       <c r="E212" s="4" t="n"/>
       <c r="F212" s="4" t="n"/>
-      <c r="H212" s="5" t="n"/>
     </row>
     <row r="213">
       <c r="E213" s="4" t="n"/>
       <c r="F213" s="4" t="n"/>
-      <c r="H213" s="5" t="n"/>
     </row>
     <row r="214">
       <c r="E214" s="4" t="n"/>
       <c r="F214" s="4" t="n"/>
-      <c r="H214" s="5" t="n"/>
     </row>
     <row r="215">
       <c r="E215" s="4" t="n"/>
       <c r="F215" s="4" t="n"/>
-      <c r="H215" s="5" t="n"/>
     </row>
     <row r="216">
       <c r="E216" s="4" t="n"/>
       <c r="F216" s="4" t="n"/>
-      <c r="H216" s="5" t="n"/>
     </row>
     <row r="217">
       <c r="E217" s="4" t="n"/>
       <c r="F217" s="4" t="n"/>
-      <c r="H217" s="5" t="n"/>
     </row>
     <row r="218">
       <c r="E218" s="4" t="n"/>
       <c r="F218" s="4" t="n"/>
-      <c r="H218" s="5" t="n"/>
     </row>
     <row r="219">
       <c r="E219" s="4" t="n"/>
       <c r="F219" s="4" t="n"/>
-      <c r="H219" s="5" t="n"/>
     </row>
     <row r="220">
       <c r="E220" s="4" t="n"/>
       <c r="F220" s="4" t="n"/>
-      <c r="H220" s="5" t="n"/>
     </row>
     <row r="221">
       <c r="E221" s="4" t="n"/>
       <c r="F221" s="4" t="n"/>
-      <c r="H221" s="5" t="n"/>
     </row>
     <row r="222">
       <c r="E222" s="4" t="n"/>
       <c r="F222" s="4" t="n"/>
-      <c r="H222" s="5" t="n"/>
     </row>
     <row r="223">
       <c r="E223" s="4" t="n"/>
       <c r="F223" s="4" t="n"/>
-      <c r="H223" s="5" t="n"/>
     </row>
     <row r="224">
       <c r="E224" s="4" t="n"/>
       <c r="F224" s="4" t="n"/>
-      <c r="H224" s="5" t="n"/>
     </row>
     <row r="225">
       <c r="E225" s="4" t="n"/>
       <c r="F225" s="4" t="n"/>
-      <c r="H225" s="5" t="n"/>
     </row>
     <row r="226">
       <c r="E226" s="4" t="n"/>
       <c r="F226" s="4" t="n"/>
-      <c r="H226" s="5" t="n"/>
     </row>
     <row r="227">
       <c r="E227" s="4" t="n"/>
       <c r="F227" s="4" t="n"/>
-      <c r="H227" s="5" t="n"/>
     </row>
     <row r="228">
       <c r="E228" s="4" t="n"/>
       <c r="F228" s="4" t="n"/>
-      <c r="H228" s="5" t="n"/>
     </row>
     <row r="229">
       <c r="E229" s="4" t="n"/>
       <c r="F229" s="4" t="n"/>
-      <c r="H229" s="5" t="n"/>
     </row>
     <row r="230">
       <c r="E230" s="4" t="n"/>
       <c r="F230" s="4" t="n"/>
-      <c r="H230" s="5" t="n"/>
     </row>
     <row r="231">
       <c r="E231" s="4" t="n"/>
       <c r="F231" s="4" t="n"/>
-      <c r="H231" s="5" t="n"/>
     </row>
     <row r="232">
       <c r="E232" s="4" t="n"/>
       <c r="F232" s="4" t="n"/>
-      <c r="H232" s="5" t="n"/>
     </row>
     <row r="233">
       <c r="E233" s="4" t="n"/>
       <c r="F233" s="4" t="n"/>
-      <c r="H233" s="5" t="n"/>
     </row>
     <row r="234">
       <c r="E234" s="4" t="n"/>
       <c r="F234" s="4" t="n"/>
-      <c r="H234" s="5" t="n"/>
     </row>
     <row r="235">
       <c r="E235" s="4" t="n"/>
       <c r="F235" s="4" t="n"/>
-      <c r="H235" s="5" t="n"/>
     </row>
     <row r="236">
       <c r="E236" s="4" t="n"/>
       <c r="F236" s="4" t="n"/>
-      <c r="H236" s="5" t="n"/>
     </row>
     <row r="237">
       <c r="E237" s="4" t="n"/>
       <c r="F237" s="4" t="n"/>
-      <c r="H237" s="5" t="n"/>
     </row>
     <row r="238">
       <c r="E238" s="4" t="n"/>
       <c r="F238" s="4" t="n"/>
-      <c r="H238" s="5" t="n"/>
     </row>
     <row r="239">
       <c r="E239" s="4" t="n"/>
       <c r="F239" s="4" t="n"/>
-      <c r="H239" s="5" t="n"/>
     </row>
     <row r="240">
       <c r="E240" s="4" t="n"/>
       <c r="F240" s="4" t="n"/>
-      <c r="H240" s="5" t="n"/>
     </row>
     <row r="241">
       <c r="E241" s="4" t="n"/>
       <c r="F241" s="4" t="n"/>
-      <c r="H241" s="5" t="n"/>
     </row>
     <row r="242">
       <c r="E242" s="4" t="n"/>
       <c r="F242" s="4" t="n"/>
-      <c r="H242" s="5" t="n"/>
     </row>
     <row r="243">
       <c r="E243" s="4" t="n"/>
       <c r="F243" s="4" t="n"/>
-      <c r="H243" s="5" t="n"/>
     </row>
     <row r="244">
       <c r="E244" s="4" t="n"/>
       <c r="F244" s="4" t="n"/>
-      <c r="H244" s="5" t="n"/>
     </row>
     <row r="245">
       <c r="E245" s="4" t="n"/>
       <c r="F245" s="4" t="n"/>
-      <c r="H245" s="5" t="n"/>
     </row>
     <row r="246">
       <c r="E246" s="4" t="n"/>
       <c r="F246" s="4" t="n"/>
-      <c r="H246" s="5" t="n"/>
     </row>
     <row r="247">
       <c r="E247" s="4" t="n"/>
       <c r="F247" s="4" t="n"/>
-      <c r="H247" s="5" t="n"/>
     </row>
     <row r="248">
       <c r="E248" s="4" t="n"/>
       <c r="F248" s="4" t="n"/>
-      <c r="H248" s="5" t="n"/>
     </row>
     <row r="249">
       <c r="E249" s="4" t="n"/>
       <c r="F249" s="4" t="n"/>
-      <c r="H249" s="5" t="n"/>
     </row>
     <row r="250">
       <c r="E250" s="4" t="n"/>
       <c r="F250" s="4" t="n"/>
-      <c r="H250" s="5" t="n"/>
     </row>
     <row r="251">
       <c r="E251" s="4" t="n"/>
       <c r="F251" s="4" t="n"/>
-      <c r="H251" s="5" t="n"/>
     </row>
     <row r="252">
       <c r="E252" s="4" t="n"/>
       <c r="F252" s="4" t="n"/>
-      <c r="H252" s="5" t="n"/>
     </row>
     <row r="253">
       <c r="E253" s="4" t="n"/>
       <c r="F253" s="4" t="n"/>
-      <c r="H253" s="5" t="n"/>
     </row>
     <row r="254">
       <c r="E254" s="4" t="n"/>
       <c r="F254" s="4" t="n"/>
-      <c r="H254" s="5" t="n"/>
     </row>
     <row r="255">
       <c r="E255" s="4" t="n"/>
       <c r="F255" s="4" t="n"/>
-      <c r="H255" s="5" t="n"/>
     </row>
     <row r="256">
       <c r="E256" s="4" t="n"/>
       <c r="F256" s="4" t="n"/>
-      <c r="H256" s="5" t="n"/>
     </row>
     <row r="257">
       <c r="E257" s="4" t="n"/>
       <c r="F257" s="4" t="n"/>
-      <c r="H257" s="5" t="n"/>
     </row>
     <row r="258">
       <c r="E258" s="4" t="n"/>
       <c r="F258" s="4" t="n"/>
-      <c r="H258" s="5" t="n"/>
     </row>
     <row r="259">
       <c r="E259" s="4" t="n"/>
       <c r="F259" s="4" t="n"/>
-      <c r="H259" s="5" t="n"/>
     </row>
     <row r="260">
       <c r="E260" s="4" t="n"/>
       <c r="F260" s="4" t="n"/>
-      <c r="H260" s="5" t="n"/>
     </row>
     <row r="261">
       <c r="E261" s="4" t="n"/>
       <c r="F261" s="4" t="n"/>
-      <c r="H261" s="5" t="n"/>
     </row>
     <row r="262">
       <c r="E262" s="4" t="n"/>
       <c r="F262" s="4" t="n"/>
-      <c r="H262" s="5" t="n"/>
     </row>
     <row r="263">
       <c r="E263" s="4" t="n"/>
       <c r="F263" s="4" t="n"/>
-      <c r="H263" s="5" t="n"/>
     </row>
     <row r="264">
       <c r="E264" s="4" t="n"/>
       <c r="F264" s="4" t="n"/>
-      <c r="H264" s="5" t="n"/>
     </row>
     <row r="265">
       <c r="E265" s="4" t="n"/>
       <c r="F265" s="4" t="n"/>
-      <c r="H265" s="5" t="n"/>
     </row>
     <row r="266">
       <c r="E266" s="4" t="n"/>
       <c r="F266" s="4" t="n"/>
-      <c r="H266" s="5" t="n"/>
     </row>
     <row r="267">
       <c r="E267" s="4" t="n"/>
       <c r="F267" s="4" t="n"/>
-      <c r="H267" s="5" t="n"/>
     </row>
     <row r="268">
       <c r="E268" s="4" t="n"/>
       <c r="F268" s="4" t="n"/>
-      <c r="H268" s="5" t="n"/>
     </row>
     <row r="269">
       <c r="E269" s="4" t="n"/>
       <c r="F269" s="4" t="n"/>
-      <c r="H269" s="5" t="n"/>
     </row>
     <row r="270">
       <c r="E270" s="4" t="n"/>
       <c r="F270" s="4" t="n"/>
-      <c r="H270" s="5" t="n"/>
     </row>
     <row r="271">
       <c r="E271" s="4" t="n"/>
       <c r="F271" s="4" t="n"/>
-      <c r="H271" s="5" t="n"/>
     </row>
     <row r="272">
       <c r="E272" s="4" t="n"/>
       <c r="F272" s="4" t="n"/>
-      <c r="H272" s="5" t="n"/>
     </row>
     <row r="273">
       <c r="E273" s="4" t="n"/>
       <c r="F273" s="4" t="n"/>
-      <c r="H273" s="5" t="n"/>
     </row>
     <row r="274">
       <c r="E274" s="4" t="n"/>
       <c r="F274" s="4" t="n"/>
-      <c r="H274" s="5" t="n"/>
     </row>
     <row r="275">
       <c r="E275" s="4" t="n"/>
       <c r="F275" s="4" t="n"/>
-      <c r="H275" s="5" t="n"/>
     </row>
     <row r="276">
       <c r="E276" s="4" t="n"/>
       <c r="F276" s="4" t="n"/>
-      <c r="H276" s="5" t="n"/>
     </row>
     <row r="277">
       <c r="E277" s="4" t="n"/>
       <c r="F277" s="4" t="n"/>
-      <c r="H277" s="5" t="n"/>
     </row>
     <row r="278">
       <c r="E278" s="4" t="n"/>
       <c r="F278" s="4" t="n"/>
-      <c r="H278" s="5" t="n"/>
     </row>
     <row r="279">
       <c r="E279" s="4" t="n"/>
       <c r="F279" s="4" t="n"/>
-      <c r="H279" s="5" t="n"/>
     </row>
     <row r="280">
       <c r="E280" s="4" t="n"/>
       <c r="F280" s="4" t="n"/>
-      <c r="H280" s="5" t="n"/>
     </row>
     <row r="281">
       <c r="E281" s="4" t="n"/>
       <c r="F281" s="4" t="n"/>
-      <c r="H281" s="5" t="n"/>
     </row>
     <row r="282">
       <c r="E282" s="4" t="n"/>
       <c r="F282" s="4" t="n"/>
-      <c r="H282" s="5" t="n"/>
     </row>
     <row r="283">
       <c r="E283" s="4" t="n"/>
       <c r="F283" s="4" t="n"/>
-      <c r="H283" s="5" t="n"/>
     </row>
     <row r="284">
       <c r="E284" s="4" t="n"/>
       <c r="F284" s="4" t="n"/>
-      <c r="H284" s="5" t="n"/>
     </row>
     <row r="285">
       <c r="E285" s="4" t="n"/>
       <c r="F285" s="4" t="n"/>
-      <c r="H285" s="5" t="n"/>
     </row>
     <row r="286">
       <c r="E286" s="4" t="n"/>
       <c r="F286" s="4" t="n"/>
-      <c r="H286" s="5" t="n"/>
     </row>
     <row r="287">
       <c r="E287" s="4" t="n"/>
       <c r="F287" s="4" t="n"/>
-      <c r="H287" s="5" t="n"/>
     </row>
     <row r="288">
       <c r="E288" s="4" t="n"/>
       <c r="F288" s="4" t="n"/>
-      <c r="H288" s="5" t="n"/>
     </row>
     <row r="289">
       <c r="E289" s="4" t="n"/>
       <c r="F289" s="4" t="n"/>
-      <c r="H289" s="5" t="n"/>
     </row>
     <row r="290">
       <c r="E290" s="4" t="n"/>
       <c r="F290" s="4" t="n"/>
-      <c r="H290" s="5" t="n"/>
     </row>
     <row r="291">
       <c r="E291" s="4" t="n"/>
       <c r="F291" s="4" t="n"/>
-      <c r="H291" s="5" t="n"/>
     </row>
     <row r="292">
       <c r="E292" s="4" t="n"/>
       <c r="F292" s="4" t="n"/>
-      <c r="H292" s="5" t="n"/>
     </row>
     <row r="293">
       <c r="E293" s="4" t="n"/>
       <c r="F293" s="4" t="n"/>
-      <c r="H293" s="5" t="n"/>
     </row>
     <row r="294">
       <c r="E294" s="4" t="n"/>
       <c r="F294" s="4" t="n"/>
-      <c r="H294" s="5" t="n"/>
     </row>
     <row r="295">
       <c r="E295" s="4" t="n"/>
       <c r="F295" s="4" t="n"/>
-      <c r="H295" s="5" t="n"/>
     </row>
     <row r="296">
       <c r="E296" s="4" t="n"/>
       <c r="F296" s="4" t="n"/>
-      <c r="H296" s="5" t="n"/>
     </row>
     <row r="297">
       <c r="E297" s="4" t="n"/>
       <c r="F297" s="4" t="n"/>
-      <c r="H297" s="5" t="n"/>
     </row>
     <row r="298">
       <c r="E298" s="4" t="n"/>
       <c r="F298" s="4" t="n"/>
-      <c r="H298" s="5" t="n"/>
     </row>
     <row r="299">
       <c r="E299" s="4" t="n"/>
       <c r="F299" s="4" t="n"/>
-      <c r="H299" s="5" t="n"/>
     </row>
     <row r="300">
       <c r="E300" s="4" t="n"/>
       <c r="F300" s="4" t="n"/>
-      <c r="H300" s="5" t="n"/>
     </row>
     <row r="301">
       <c r="E301" s="4" t="n"/>
       <c r="F301" s="4" t="n"/>
-      <c r="H301" s="5" t="n"/>
     </row>
     <row r="302">
       <c r="E302" s="4" t="n"/>
       <c r="F302" s="4" t="n"/>
-      <c r="H302" s="5" t="n"/>
     </row>
     <row r="303">
       <c r="E303" s="4" t="n"/>
       <c r="F303" s="4" t="n"/>
-      <c r="H303" s="5" t="n"/>
     </row>
     <row r="304">
       <c r="E304" s="4" t="n"/>
       <c r="F304" s="4" t="n"/>
-      <c r="H304" s="5" t="n"/>
     </row>
     <row r="305">
       <c r="E305" s="4" t="n"/>
       <c r="F305" s="4" t="n"/>
-      <c r="H305" s="5" t="n"/>
     </row>
     <row r="306">
       <c r="E306" s="4" t="n"/>
       <c r="F306" s="4" t="n"/>
-      <c r="H306" s="5" t="n"/>
     </row>
     <row r="307">
       <c r="E307" s="4" t="n"/>
       <c r="F307" s="4" t="n"/>
-      <c r="H307" s="5" t="n"/>
     </row>
     <row r="308">
       <c r="E308" s="4" t="n"/>
       <c r="F308" s="4" t="n"/>
-      <c r="H308" s="5" t="n"/>
     </row>
     <row r="309">
       <c r="E309" s="4" t="n"/>
       <c r="F309" s="4" t="n"/>
-      <c r="H309" s="5" t="n"/>
     </row>
     <row r="310">
       <c r="E310" s="4" t="n"/>
       <c r="F310" s="4" t="n"/>
-      <c r="H310" s="5" t="n"/>
     </row>
     <row r="311">
       <c r="E311" s="4" t="n"/>
       <c r="F311" s="4" t="n"/>
-      <c r="H311" s="5" t="n"/>
     </row>
     <row r="312">
       <c r="E312" s="4" t="n"/>
       <c r="F312" s="4" t="n"/>
-      <c r="H312" s="5" t="n"/>
     </row>
     <row r="313">
       <c r="E313" s="4" t="n"/>
       <c r="F313" s="4" t="n"/>
-      <c r="H313" s="5" t="n"/>
     </row>
     <row r="314">
       <c r="E314" s="4" t="n"/>
       <c r="F314" s="4" t="n"/>
-      <c r="H314" s="5" t="n"/>
     </row>
     <row r="315">
       <c r="E315" s="4" t="n"/>
       <c r="F315" s="4" t="n"/>
-      <c r="H315" s="5" t="n"/>
     </row>
     <row r="316">
       <c r="E316" s="4" t="n"/>
       <c r="F316" s="4" t="n"/>
-      <c r="H316" s="5" t="n"/>
     </row>
     <row r="317">
       <c r="E317" s="4" t="n"/>
       <c r="F317" s="4" t="n"/>
-      <c r="H317" s="5" t="n"/>
     </row>
     <row r="318">
       <c r="E318" s="4" t="n"/>
       <c r="F318" s="4" t="n"/>
-      <c r="H318" s="5" t="n"/>
     </row>
     <row r="319">
       <c r="E319" s="4" t="n"/>
       <c r="F319" s="4" t="n"/>
-      <c r="H319" s="5" t="n"/>
     </row>
     <row r="320">
       <c r="E320" s="4" t="n"/>
       <c r="F320" s="4" t="n"/>
-      <c r="H320" s="5" t="n"/>
     </row>
     <row r="321">
       <c r="E321" s="4" t="n"/>
       <c r="F321" s="4" t="n"/>
-      <c r="H321" s="5" t="n"/>
     </row>
     <row r="322">
       <c r="E322" s="4" t="n"/>
       <c r="F322" s="4" t="n"/>
-      <c r="H322" s="5" t="n"/>
     </row>
     <row r="323">
       <c r="E323" s="4" t="n"/>
       <c r="F323" s="4" t="n"/>
-      <c r="H323" s="5" t="n"/>
     </row>
     <row r="324">
       <c r="E324" s="4" t="n"/>
       <c r="F324" s="4" t="n"/>
-      <c r="H324" s="5" t="n"/>
     </row>
     <row r="325">
       <c r="E325" s="4" t="n"/>
       <c r="F325" s="4" t="n"/>
-      <c r="H325" s="5" t="n"/>
     </row>
     <row r="326">
       <c r="E326" s="4" t="n"/>
       <c r="F326" s="4" t="n"/>
-      <c r="H326" s="5" t="n"/>
     </row>
     <row r="327">
       <c r="E327" s="4" t="n"/>
       <c r="F327" s="4" t="n"/>
-      <c r="H327" s="5" t="n"/>
     </row>
     <row r="328">
       <c r="E328" s="4" t="n"/>
       <c r="F328" s="4" t="n"/>
-      <c r="H328" s="5" t="n"/>
     </row>
     <row r="329">
       <c r="E329" s="4" t="n"/>
       <c r="F329" s="4" t="n"/>
-      <c r="H329" s="5" t="n"/>
     </row>
     <row r="330">
       <c r="E330" s="4" t="n"/>
       <c r="F330" s="4" t="n"/>
-      <c r="H330" s="5" t="n"/>
     </row>
     <row r="331">
       <c r="E331" s="4" t="n"/>
       <c r="F331" s="4" t="n"/>
-      <c r="H331" s="5" t="n"/>
     </row>
     <row r="332">
       <c r="E332" s="4" t="n"/>
       <c r="F332" s="4" t="n"/>
-      <c r="H332" s="5" t="n"/>
     </row>
     <row r="333">
       <c r="E333" s="4" t="n"/>
       <c r="F333" s="4" t="n"/>
-      <c r="H333" s="5" t="n"/>
     </row>
     <row r="334">
       <c r="E334" s="4" t="n"/>
       <c r="F334" s="4" t="n"/>
-      <c r="H334" s="5" t="n"/>
     </row>
     <row r="335">
       <c r="E335" s="4" t="n"/>
       <c r="F335" s="4" t="n"/>
-      <c r="H335" s="5" t="n"/>
     </row>
     <row r="336">
       <c r="E336" s="4" t="n"/>
       <c r="F336" s="4" t="n"/>
-      <c r="H336" s="5" t="n"/>
     </row>
     <row r="337">
       <c r="E337" s="4" t="n"/>
       <c r="F337" s="4" t="n"/>
-      <c r="H337" s="5" t="n"/>
     </row>
     <row r="338">
       <c r="E338" s="4" t="n"/>
       <c r="F338" s="4" t="n"/>
-      <c r="H338" s="5" t="n"/>
     </row>
     <row r="339">
       <c r="E339" s="4" t="n"/>
       <c r="F339" s="4" t="n"/>
-      <c r="H339" s="5" t="n"/>
     </row>
     <row r="340">
       <c r="E340" s="4" t="n"/>
       <c r="F340" s="4" t="n"/>
-      <c r="H340" s="5" t="n"/>
     </row>
     <row r="341">
       <c r="E341" s="4" t="n"/>
       <c r="F341" s="4" t="n"/>
-      <c r="H341" s="5" t="n"/>
     </row>
     <row r="342">
       <c r="E342" s="4" t="n"/>
       <c r="F342" s="4" t="n"/>
-      <c r="H342" s="5" t="n"/>
     </row>
     <row r="343">
       <c r="E343" s="4" t="n"/>
       <c r="F343" s="4" t="n"/>
-      <c r="H343" s="5" t="n"/>
     </row>
     <row r="344">
       <c r="E344" s="4" t="n"/>
       <c r="F344" s="4" t="n"/>
-      <c r="H344" s="5" t="n"/>
     </row>
     <row r="345">
       <c r="E345" s="4" t="n"/>
       <c r="F345" s="4" t="n"/>
-      <c r="H345" s="5" t="n"/>
     </row>
     <row r="346">
       <c r="E346" s="4" t="n"/>
       <c r="F346" s="4" t="n"/>
-      <c r="H346" s="5" t="n"/>
     </row>
     <row r="347">
       <c r="E347" s="4" t="n"/>
       <c r="F347" s="4" t="n"/>
-      <c r="H347" s="5" t="n"/>
     </row>
     <row r="348">
       <c r="E348" s="4" t="n"/>
       <c r="F348" s="4" t="n"/>
-      <c r="H348" s="5" t="n"/>
     </row>
     <row r="349">
       <c r="E349" s="4" t="n"/>
       <c r="F349" s="4" t="n"/>
-      <c r="H349" s="5" t="n"/>
     </row>
     <row r="350">
       <c r="E350" s="4" t="n"/>
       <c r="F350" s="4" t="n"/>
-      <c r="H350" s="5" t="n"/>
     </row>
     <row r="351">
       <c r="E351" s="4" t="n"/>
       <c r="F351" s="4" t="n"/>
-      <c r="H351" s="5" t="n"/>
     </row>
     <row r="352">
       <c r="E352" s="4" t="n"/>
       <c r="F352" s="4" t="n"/>
-      <c r="H352" s="5" t="n"/>
     </row>
     <row r="353">
       <c r="E353" s="4" t="n"/>
       <c r="F353" s="4" t="n"/>
-      <c r="H353" s="5" t="n"/>
     </row>
     <row r="354">
       <c r="E354" s="4" t="n"/>
       <c r="F354" s="4" t="n"/>
-      <c r="H354" s="5" t="n"/>
     </row>
     <row r="355">
       <c r="E355" s="4" t="n"/>
       <c r="F355" s="4" t="n"/>
-      <c r="H355" s="5" t="n"/>
     </row>
     <row r="356">
       <c r="E356" s="4" t="n"/>
       <c r="F356" s="4" t="n"/>
-      <c r="H356" s="5" t="n"/>
     </row>
     <row r="357">
       <c r="E357" s="4" t="n"/>
       <c r="F357" s="4" t="n"/>
-      <c r="H357" s="5" t="n"/>
     </row>
     <row r="358">
       <c r="E358" s="4" t="n"/>
       <c r="F358" s="4" t="n"/>
-      <c r="H358" s="5" t="n"/>
     </row>
     <row r="359">
       <c r="E359" s="4" t="n"/>
       <c r="F359" s="4" t="n"/>
-      <c r="H359" s="5" t="n"/>
     </row>
     <row r="360">
       <c r="E360" s="4" t="n"/>
       <c r="F360" s="4" t="n"/>
-      <c r="H360" s="5" t="n"/>
     </row>
     <row r="361">
       <c r="E361" s="4" t="n"/>
       <c r="F361" s="4" t="n"/>
-      <c r="H361" s="5" t="n"/>
     </row>
     <row r="362">
       <c r="E362" s="4" t="n"/>
       <c r="F362" s="4" t="n"/>
-      <c r="H362" s="5" t="n"/>
     </row>
     <row r="363">
       <c r="E363" s="4" t="n"/>
       <c r="F363" s="4" t="n"/>
-      <c r="H363" s="5" t="n"/>
     </row>
     <row r="364">
       <c r="E364" s="4" t="n"/>
       <c r="F364" s="4" t="n"/>
-      <c r="H364" s="5" t="n"/>
     </row>
     <row r="365">
       <c r="E365" s="4" t="n"/>
       <c r="F365" s="4" t="n"/>
-      <c r="H365" s="5" t="n"/>
     </row>
     <row r="366">
       <c r="E366" s="4" t="n"/>
       <c r="F366" s="4" t="n"/>
-      <c r="H366" s="5" t="n"/>
     </row>
     <row r="367">
       <c r="E367" s="4" t="n"/>
       <c r="F367" s="4" t="n"/>
-      <c r="H367" s="5" t="n"/>
     </row>
     <row r="368">
       <c r="E368" s="4" t="n"/>
       <c r="F368" s="4" t="n"/>
-      <c r="H368" s="5" t="n"/>
     </row>
     <row r="369">
       <c r="E369" s="4" t="n"/>
       <c r="F369" s="4" t="n"/>
-      <c r="H369" s="5" t="n"/>
     </row>
     <row r="370">
       <c r="E370" s="4" t="n"/>
       <c r="F370" s="4" t="n"/>
-      <c r="H370" s="5" t="n"/>
     </row>
     <row r="371">
       <c r="E371" s="4" t="n"/>
       <c r="F371" s="4" t="n"/>
-      <c r="H371" s="5" t="n"/>
     </row>
     <row r="372">
       <c r="E372" s="4" t="n"/>
       <c r="F372" s="4" t="n"/>
-      <c r="H372" s="5" t="n"/>
     </row>
     <row r="373">
       <c r="E373" s="4" t="n"/>
       <c r="F373" s="4" t="n"/>
-      <c r="H373" s="5" t="n"/>
     </row>
     <row r="374">
       <c r="E374" s="4" t="n"/>
       <c r="F374" s="4" t="n"/>
-      <c r="H374" s="5" t="n"/>
     </row>
     <row r="375">
       <c r="E375" s="4" t="n"/>
       <c r="F375" s="4" t="n"/>
-      <c r="H375" s="5" t="n"/>
     </row>
     <row r="376">
       <c r="E376" s="4" t="n"/>
       <c r="F376" s="4" t="n"/>
-      <c r="H376" s="5" t="n"/>
     </row>
     <row r="377">
       <c r="E377" s="4" t="n"/>
       <c r="F377" s="4" t="n"/>
-      <c r="H377" s="5" t="n"/>
     </row>
     <row r="378">
       <c r="E378" s="4" t="n"/>
       <c r="F378" s="4" t="n"/>
-      <c r="H378" s="5" t="n"/>
     </row>
     <row r="379">
       <c r="E379" s="4" t="n"/>
       <c r="F379" s="4" t="n"/>
-      <c r="H379" s="5" t="n"/>
     </row>
     <row r="380">
       <c r="E380" s="4" t="n"/>
       <c r="F380" s="4" t="n"/>
-      <c r="H380" s="5" t="n"/>
     </row>
     <row r="381">
       <c r="E381" s="4" t="n"/>
       <c r="F381" s="4" t="n"/>
-      <c r="H381" s="5" t="n"/>
     </row>
     <row r="382">
       <c r="E382" s="4" t="n"/>
       <c r="F382" s="4" t="n"/>
-      <c r="H382" s="5" t="n"/>
     </row>
     <row r="383">
       <c r="E383" s="4" t="n"/>
       <c r="F383" s="4" t="n"/>
-      <c r="H383" s="5" t="n"/>
     </row>
     <row r="384">
       <c r="E384" s="4" t="n"/>
       <c r="F384" s="4" t="n"/>
-      <c r="H384" s="5" t="n"/>
     </row>
     <row r="385">
       <c r="E385" s="4" t="n"/>
       <c r="F385" s="4" t="n"/>
-      <c r="H385" s="5" t="n"/>
     </row>
     <row r="386">
       <c r="E386" s="4" t="n"/>
       <c r="F386" s="4" t="n"/>
-      <c r="H386" s="5" t="n"/>
     </row>
     <row r="387">
       <c r="E387" s="4" t="n"/>
       <c r="F387" s="4" t="n"/>
-      <c r="H387" s="5" t="n"/>
     </row>
     <row r="388">
       <c r="E388" s="4" t="n"/>
       <c r="F388" s="4" t="n"/>
-      <c r="H388" s="5" t="n"/>
     </row>
     <row r="389">
       <c r="E389" s="4" t="n"/>
       <c r="F389" s="4" t="n"/>
-      <c r="H389" s="5" t="n"/>
     </row>
     <row r="390">
       <c r="E390" s="4" t="n"/>
       <c r="F390" s="4" t="n"/>
-      <c r="H390" s="5" t="n"/>
     </row>
     <row r="391">
       <c r="E391" s="4" t="n"/>
       <c r="F391" s="4" t="n"/>
-      <c r="H391" s="5" t="n"/>
     </row>
     <row r="392">
       <c r="E392" s="4" t="n"/>
       <c r="F392" s="4" t="n"/>
-      <c r="H392" s="5" t="n"/>
     </row>
     <row r="393">
       <c r="E393" s="4" t="n"/>
       <c r="F393" s="4" t="n"/>
-      <c r="H393" s="5" t="n"/>
     </row>
     <row r="394">
       <c r="E394" s="4" t="n"/>
       <c r="F394" s="4" t="n"/>
-      <c r="H394" s="5" t="n"/>
     </row>
     <row r="395">
       <c r="E395" s="4" t="n"/>
       <c r="F395" s="4" t="n"/>
-      <c r="H395" s="5" t="n"/>
     </row>
     <row r="396">
       <c r="E396" s="4" t="n"/>
       <c r="F396" s="4" t="n"/>
-      <c r="H396" s="5" t="n"/>
     </row>
     <row r="397">
       <c r="E397" s="4" t="n"/>
       <c r="F397" s="4" t="n"/>
-      <c r="H397" s="5" t="n"/>
     </row>
     <row r="398">
       <c r="E398" s="4" t="n"/>
       <c r="F398" s="4" t="n"/>
-      <c r="H398" s="5" t="n"/>
     </row>
     <row r="399">
       <c r="E399" s="4" t="n"/>
       <c r="F399" s="4" t="n"/>
-      <c r="H399" s="5" t="n"/>
     </row>
     <row r="400">
       <c r="E400" s="4" t="n"/>
       <c r="F400" s="4" t="n"/>
-      <c r="H400" s="5" t="n"/>
     </row>
     <row r="401">
       <c r="E401" s="4" t="n"/>
       <c r="F401" s="4" t="n"/>
-      <c r="H401" s="5" t="n"/>
     </row>
     <row r="402">
       <c r="E402" s="4" t="n"/>
       <c r="F402" s="4" t="n"/>
-      <c r="H402" s="5" t="n"/>
     </row>
     <row r="403">
       <c r="E403" s="4" t="n"/>
       <c r="F403" s="4" t="n"/>
-      <c r="H403" s="5" t="n"/>
     </row>
     <row r="404">
       <c r="E404" s="4" t="n"/>
       <c r="F404" s="4" t="n"/>
-      <c r="H404" s="5" t="n"/>
     </row>
     <row r="405">
       <c r="E405" s="4" t="n"/>
       <c r="F405" s="4" t="n"/>
-      <c r="H405" s="5" t="n"/>
     </row>
     <row r="406">
       <c r="E406" s="4" t="n"/>
       <c r="F406" s="4" t="n"/>
-      <c r="H406" s="5" t="n"/>
     </row>
     <row r="407">
       <c r="E407" s="4" t="n"/>
       <c r="F407" s="4" t="n"/>
-      <c r="H407" s="5" t="n"/>
     </row>
     <row r="408">
       <c r="E408" s="4" t="n"/>
       <c r="F408" s="4" t="n"/>
-      <c r="H408" s="5" t="n"/>
     </row>
     <row r="409">
       <c r="E409" s="4" t="n"/>
       <c r="F409" s="4" t="n"/>
-      <c r="H409" s="5" t="n"/>
     </row>
     <row r="410">
       <c r="E410" s="4" t="n"/>
       <c r="F410" s="4" t="n"/>
-      <c r="H410" s="5" t="n"/>
     </row>
     <row r="411">
       <c r="E411" s="4" t="n"/>
       <c r="F411" s="4" t="n"/>
-      <c r="H411" s="5" t="n"/>
     </row>
     <row r="412">
       <c r="E412" s="4" t="n"/>
       <c r="F412" s="4" t="n"/>
-      <c r="H412" s="5" t="n"/>
     </row>
     <row r="413">
       <c r="E413" s="4" t="n"/>
       <c r="F413" s="4" t="n"/>
-      <c r="H413" s="5" t="n"/>
     </row>
     <row r="414">
       <c r="E414" s="4" t="n"/>
       <c r="F414" s="4" t="n"/>
-      <c r="H414" s="5" t="n"/>
     </row>
     <row r="415">
       <c r="E415" s="4" t="n"/>
       <c r="F415" s="4" t="n"/>
-      <c r="H415" s="5" t="n"/>
     </row>
     <row r="416">
       <c r="E416" s="4" t="n"/>
       <c r="F416" s="4" t="n"/>
-      <c r="H416" s="5" t="n"/>
     </row>
     <row r="417">
       <c r="E417" s="4" t="n"/>
       <c r="F417" s="4" t="n"/>
-      <c r="H417" s="5" t="n"/>
     </row>
     <row r="418">
       <c r="E418" s="4" t="n"/>
       <c r="F418" s="4" t="n"/>
-      <c r="H418" s="5" t="n"/>
     </row>
     <row r="419">
       <c r="E419" s="4" t="n"/>
       <c r="F419" s="4" t="n"/>
-      <c r="H419" s="5" t="n"/>
     </row>
     <row r="420">
       <c r="E420" s="4" t="n"/>
       <c r="F420" s="4" t="n"/>
-      <c r="H420" s="5" t="n"/>
     </row>
     <row r="421">
       <c r="E421" s="4" t="n"/>
       <c r="F421" s="4" t="n"/>
-      <c r="H421" s="5" t="n"/>
     </row>
     <row r="422">
       <c r="E422" s="4" t="n"/>
       <c r="F422" s="4" t="n"/>
-      <c r="H422" s="5" t="n"/>
     </row>
     <row r="423">
       <c r="E423" s="4" t="n"/>
       <c r="F423" s="4" t="n"/>
-      <c r="H423" s="5" t="n"/>
     </row>
     <row r="424">
       <c r="E424" s="4" t="n"/>
       <c r="F424" s="4" t="n"/>
-      <c r="H424" s="5" t="n"/>
     </row>
     <row r="425">
       <c r="E425" s="4" t="n"/>
       <c r="F425" s="4" t="n"/>
-      <c r="H425" s="5" t="n"/>
     </row>
     <row r="426">
       <c r="E426" s="4" t="n"/>
       <c r="F426" s="4" t="n"/>
-      <c r="H426" s="5" t="n"/>
     </row>
     <row r="427">
       <c r="E427" s="4" t="n"/>
       <c r="F427" s="4" t="n"/>
-      <c r="H427" s="5" t="n"/>
     </row>
     <row r="428">
       <c r="E428" s="4" t="n"/>
       <c r="F428" s="4" t="n"/>
-      <c r="H428" s="5" t="n"/>
     </row>
     <row r="429">
       <c r="E429" s="4" t="n"/>
       <c r="F429" s="4" t="n"/>
-      <c r="H429" s="5" t="n"/>
     </row>
     <row r="430">
       <c r="E430" s="4" t="n"/>
       <c r="F430" s="4" t="n"/>
-      <c r="H430" s="5" t="n"/>
     </row>
     <row r="431">
       <c r="E431" s="4" t="n"/>
       <c r="F431" s="4" t="n"/>
-      <c r="H431" s="5" t="n"/>
     </row>
     <row r="432">
       <c r="E432" s="4" t="n"/>
       <c r="F432" s="4" t="n"/>
-      <c r="H432" s="5" t="n"/>
     </row>
     <row r="433">
       <c r="E433" s="4" t="n"/>
       <c r="F433" s="4" t="n"/>
-      <c r="H433" s="5" t="n"/>
     </row>
     <row r="434">
       <c r="E434" s="4" t="n"/>
       <c r="F434" s="4" t="n"/>
-      <c r="H434" s="5" t="n"/>
     </row>
     <row r="435">
       <c r="E435" s="4" t="n"/>
       <c r="F435" s="4" t="n"/>
-      <c r="H435" s="5" t="n"/>
     </row>
     <row r="436">
       <c r="E436" s="4" t="n"/>
       <c r="F436" s="4" t="n"/>
-      <c r="H436" s="5" t="n"/>
     </row>
     <row r="437">
       <c r="E437" s="4" t="n"/>
       <c r="F437" s="4" t="n"/>
-      <c r="H437" s="5" t="n"/>
     </row>
     <row r="438">
       <c r="E438" s="4" t="n"/>
       <c r="F438" s="4" t="n"/>
-      <c r="H438" s="5" t="n"/>
     </row>
     <row r="439">
       <c r="E439" s="4" t="n"/>
       <c r="F439" s="4" t="n"/>
-      <c r="H439" s="5" t="n"/>
     </row>
     <row r="440">
       <c r="E440" s="4" t="n"/>
       <c r="F440" s="4" t="n"/>
-      <c r="H440" s="5" t="n"/>
     </row>
     <row r="441">
       <c r="E441" s="4" t="n"/>
       <c r="F441" s="4" t="n"/>
-      <c r="H441" s="5" t="n"/>
     </row>
     <row r="442">
       <c r="E442" s="4" t="n"/>
       <c r="F442" s="4" t="n"/>
-      <c r="H442" s="5" t="n"/>
     </row>
     <row r="443">
       <c r="E443" s="4" t="n"/>
       <c r="F443" s="4" t="n"/>
-      <c r="H443" s="5" t="n"/>
     </row>
     <row r="444">
       <c r="E444" s="4" t="n"/>
       <c r="F444" s="4" t="n"/>
-      <c r="H444" s="5" t="n"/>
     </row>
     <row r="445">
       <c r="E445" s="4" t="n"/>
       <c r="F445" s="4" t="n"/>
-      <c r="H445" s="5" t="n"/>
     </row>
     <row r="446">
       <c r="E446" s="4" t="n"/>
       <c r="F446" s="4" t="n"/>
-      <c r="H446" s="5" t="n"/>
     </row>
     <row r="447">
       <c r="E447" s="4" t="n"/>
       <c r="F447" s="4" t="n"/>
-      <c r="H447" s="5" t="n"/>
     </row>
     <row r="448">
       <c r="E448" s="4" t="n"/>
       <c r="F448" s="4" t="n"/>
-      <c r="H448" s="5" t="n"/>
     </row>
     <row r="449">
       <c r="E449" s="4" t="n"/>
       <c r="F449" s="4" t="n"/>
-      <c r="H449" s="5" t="n"/>
     </row>
     <row r="450">
       <c r="E450" s="4" t="n"/>
       <c r="F450" s="4" t="n"/>
-      <c r="H450" s="5" t="n"/>
     </row>
     <row r="451">
       <c r="E451" s="4" t="n"/>
       <c r="F451" s="4" t="n"/>
-      <c r="H451" s="5" t="n"/>
     </row>
     <row r="452">
       <c r="E452" s="4" t="n"/>
       <c r="F452" s="4" t="n"/>
-      <c r="H452" s="5" t="n"/>
     </row>
     <row r="453">
       <c r="E453" s="4" t="n"/>
       <c r="F453" s="4" t="n"/>
-      <c r="H453" s="5" t="n"/>
     </row>
     <row r="454">
       <c r="E454" s="4" t="n"/>
       <c r="F454" s="4" t="n"/>
-      <c r="H454" s="5" t="n"/>
     </row>
     <row r="455">
       <c r="E455" s="4" t="n"/>
       <c r="F455" s="4" t="n"/>
-      <c r="H455" s="5" t="n"/>
     </row>
     <row r="456">
       <c r="E456" s="4" t="n"/>
       <c r="F456" s="4" t="n"/>
-      <c r="H456" s="5" t="n"/>
     </row>
     <row r="457">
       <c r="E457" s="4" t="n"/>
       <c r="F457" s="4" t="n"/>
-      <c r="H457" s="5" t="n"/>
     </row>
     <row r="458">
       <c r="E458" s="4" t="n"/>
       <c r="F458" s="4" t="n"/>
-      <c r="H458" s="5" t="n"/>
     </row>
     <row r="459">
       <c r="E459" s="4" t="n"/>
       <c r="F459" s="4" t="n"/>
-      <c r="H459" s="5" t="n"/>
     </row>
     <row r="460">
       <c r="E460" s="4" t="n"/>
       <c r="F460" s="4" t="n"/>
-      <c r="H460" s="5" t="n"/>
     </row>
     <row r="461">
       <c r="E461" s="4" t="n"/>
       <c r="F461" s="4" t="n"/>
-      <c r="H461" s="5" t="n"/>
     </row>
     <row r="462">
       <c r="E462" s="4" t="n"/>
       <c r="F462" s="4" t="n"/>
-      <c r="H462" s="5" t="n"/>
     </row>
     <row r="463">
       <c r="E463" s="4" t="n"/>
       <c r="F463" s="4" t="n"/>
-      <c r="H463" s="5" t="n"/>
     </row>
     <row r="464">
       <c r="E464" s="4" t="n"/>
       <c r="F464" s="4" t="n"/>
-      <c r="H464" s="5" t="n"/>
     </row>
     <row r="465">
       <c r="E465" s="4" t="n"/>
       <c r="F465" s="4" t="n"/>
-      <c r="H465" s="5" t="n"/>
     </row>
     <row r="466">
       <c r="E466" s="4" t="n"/>
       <c r="F466" s="4" t="n"/>
-      <c r="H466" s="5" t="n"/>
     </row>
     <row r="467">
       <c r="E467" s="4" t="n"/>
       <c r="F467" s="4" t="n"/>
-      <c r="H467" s="5" t="n"/>
     </row>
     <row r="468">
       <c r="E468" s="4" t="n"/>
       <c r="F468" s="4" t="n"/>
-      <c r="H468" s="5" t="n"/>
     </row>
     <row r="469">
       <c r="E469" s="4" t="n"/>
       <c r="F469" s="4" t="n"/>
-      <c r="H469" s="5" t="n"/>
     </row>
     <row r="470">
       <c r="E470" s="4" t="n"/>
       <c r="F470" s="4" t="n"/>
-      <c r="H470" s="5" t="n"/>
     </row>
     <row r="471">
       <c r="E471" s="4" t="n"/>
       <c r="F471" s="4" t="n"/>
-      <c r="H471" s="5" t="n"/>
     </row>
     <row r="472">
       <c r="E472" s="4" t="n"/>
       <c r="F472" s="4" t="n"/>
-      <c r="H472" s="5" t="n"/>
     </row>
     <row r="473">
       <c r="E473" s="4" t="n"/>
       <c r="F473" s="4" t="n"/>
-      <c r="H473" s="5" t="n"/>
     </row>
     <row r="474">
       <c r="E474" s="4" t="n"/>
       <c r="F474" s="4" t="n"/>
-      <c r="H474" s="5" t="n"/>
     </row>
     <row r="475">
       <c r="E475" s="4" t="n"/>
       <c r="F475" s="4" t="n"/>
-      <c r="H475" s="5" t="n"/>
     </row>
     <row r="476">
       <c r="E476" s="4" t="n"/>
       <c r="F476" s="4" t="n"/>
-      <c r="H476" s="5" t="n"/>
     </row>
     <row r="477">
       <c r="E477" s="4" t="n"/>
       <c r="F477" s="4" t="n"/>
-      <c r="H477" s="5" t="n"/>
     </row>
     <row r="478">
       <c r="E478" s="4" t="n"/>
       <c r="F478" s="4" t="n"/>
-      <c r="H478" s="5" t="n"/>
     </row>
     <row r="479">
       <c r="E479" s="4" t="n"/>
       <c r="F479" s="4" t="n"/>
-      <c r="H479" s="5" t="n"/>
     </row>
     <row r="480">
       <c r="E480" s="4" t="n"/>
       <c r="F480" s="4" t="n"/>
-      <c r="H480" s="5" t="n"/>
     </row>
     <row r="481">
       <c r="E481" s="4" t="n"/>
       <c r="F481" s="4" t="n"/>
-      <c r="H481" s="5" t="n"/>
     </row>
     <row r="482">
       <c r="E482" s="4" t="n"/>
       <c r="F482" s="4" t="n"/>
-      <c r="H482" s="5" t="n"/>
     </row>
     <row r="483">
       <c r="E483" s="4" t="n"/>
       <c r="F483" s="4" t="n"/>
-      <c r="H483" s="5" t="n"/>
     </row>
     <row r="484">
       <c r="E484" s="4" t="n"/>
       <c r="F484" s="4" t="n"/>
-      <c r="H484" s="5" t="n"/>
     </row>
     <row r="485">
       <c r="E485" s="4" t="n"/>
       <c r="F485" s="4" t="n"/>
-      <c r="H485" s="5" t="n"/>
     </row>
     <row r="486">
       <c r="E486" s="4" t="n"/>
       <c r="F486" s="4" t="n"/>
-      <c r="H486" s="5" t="n"/>
     </row>
     <row r="487">
       <c r="E487" s="4" t="n"/>
       <c r="F487" s="4" t="n"/>
-      <c r="H487" s="5" t="n"/>
     </row>
     <row r="488">
       <c r="E488" s="4" t="n"/>
       <c r="F488" s="4" t="n"/>
-      <c r="H488" s="5" t="n"/>
     </row>
     <row r="489">
       <c r="E489" s="4" t="n"/>
       <c r="F489" s="4" t="n"/>
-      <c r="H489" s="5" t="n"/>
     </row>
     <row r="490">
       <c r="E490" s="4" t="n"/>
       <c r="F490" s="4" t="n"/>
-      <c r="H490" s="5" t="n"/>
     </row>
     <row r="491">
       <c r="E491" s="4" t="n"/>
       <c r="F491" s="4" t="n"/>
-      <c r="H491" s="5" t="n"/>
     </row>
     <row r="492">
       <c r="E492" s="4" t="n"/>
       <c r="F492" s="4" t="n"/>
-      <c r="H492" s="5" t="n"/>
     </row>
     <row r="493">
       <c r="E493" s="4" t="n"/>
       <c r="F493" s="4" t="n"/>
-      <c r="H493" s="5" t="n"/>
     </row>
     <row r="494">
       <c r="E494" s="4" t="n"/>
       <c r="F494" s="4" t="n"/>
-      <c r="H494" s="5" t="n"/>
     </row>
     <row r="495">
       <c r="E495" s="4" t="n"/>
       <c r="F495" s="4" t="n"/>
-      <c r="H495" s="5" t="n"/>
     </row>
     <row r="496">
       <c r="E496" s="4" t="n"/>
       <c r="F496" s="4" t="n"/>
-      <c r="H496" s="5" t="n"/>
     </row>
     <row r="497">
       <c r="E497" s="4" t="n"/>
       <c r="F497" s="4" t="n"/>
-      <c r="H497" s="5" t="n"/>
     </row>
     <row r="498">
       <c r="E498" s="4" t="n"/>
       <c r="F498" s="4" t="n"/>
-      <c r="H498" s="5" t="n"/>
     </row>
     <row r="499">
       <c r="E499" s="4" t="n"/>
       <c r="F499" s="4" t="n"/>
-      <c r="H499" s="5" t="n"/>
     </row>
     <row r="500">
       <c r="E500" s="4" t="n"/>
       <c r="F500" s="4" t="n"/>
-      <c r="H500" s="5" t="n"/>
     </row>
   </sheetData>
   <dataValidations count="3">
@@ -3566,6 +3063,2073 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:D500"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="40" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="3" t="inlineStr">
+        <is>
+          <t>id_implantacao</t>
+        </is>
+      </c>
+      <c r="B1" s="3" t="inlineStr">
+        <is>
+          <t>categoria</t>
+        </is>
+      </c>
+      <c r="C1" s="3" t="inlineStr">
+        <is>
+          <t>valor_provisionado</t>
+        </is>
+      </c>
+      <c r="D1" s="3" t="inlineStr">
+        <is>
+          <t>observacao</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>IMP-001</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Equipamentos/materiais</t>
+        </is>
+      </c>
+      <c r="C2" s="5" t="n">
+        <v>26900</v>
+      </c>
+      <c r="D2" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>IMP-001</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Mão de obra própria</t>
+        </is>
+      </c>
+      <c r="C3" s="5" t="n">
+        <v>10100</v>
+      </c>
+      <c r="D3" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>IMP-001</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Terceiros/empreiteiros</t>
+        </is>
+      </c>
+      <c r="C4" s="5" t="n">
+        <v>8600</v>
+      </c>
+      <c r="D4" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>IMP-001</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Deslocamento/infraestrutura</t>
+        </is>
+      </c>
+      <c r="C5" s="5" t="n">
+        <v>2400</v>
+      </c>
+      <c r="D5" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>IMP-002</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Equipamentos/materiais</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="n">
+        <v>17600</v>
+      </c>
+      <c r="D6" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>IMP-002</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Mão de obra própria</t>
+        </is>
+      </c>
+      <c r="C7" s="5" t="n">
+        <v>6600</v>
+      </c>
+      <c r="D7" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>IMP-002</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Terceiros/empreiteiros</t>
+        </is>
+      </c>
+      <c r="C8" s="5" t="n">
+        <v>5700</v>
+      </c>
+      <c r="D8" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>IMP-002</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Deslocamento/infraestrutura</t>
+        </is>
+      </c>
+      <c r="C9" s="5" t="n">
+        <v>1600</v>
+      </c>
+      <c r="D9" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>IMP-003</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Equipamentos/materiais</t>
+        </is>
+      </c>
+      <c r="C10" s="5" t="n">
+        <v>12800</v>
+      </c>
+      <c r="D10" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>IMP-003</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Mão de obra própria</t>
+        </is>
+      </c>
+      <c r="C11" s="5" t="n">
+        <v>4800</v>
+      </c>
+      <c r="D11" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>IMP-003</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Terceiros/empreiteiros</t>
+        </is>
+      </c>
+      <c r="C12" s="5" t="n">
+        <v>4100</v>
+      </c>
+      <c r="D12" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>IMP-003</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Deslocamento/infraestrutura</t>
+        </is>
+      </c>
+      <c r="C13" s="5" t="n">
+        <v>1100</v>
+      </c>
+      <c r="D13" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>IMP-004</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Equipamentos/materiais</t>
+        </is>
+      </c>
+      <c r="C14" s="5" t="n">
+        <v>15000</v>
+      </c>
+      <c r="D14" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>IMP-004</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Mão de obra própria</t>
+        </is>
+      </c>
+      <c r="C15" s="5" t="n">
+        <v>5600</v>
+      </c>
+      <c r="D15" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>IMP-004</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Terceiros/empreiteiros</t>
+        </is>
+      </c>
+      <c r="C16" s="5" t="n">
+        <v>4800</v>
+      </c>
+      <c r="D16" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>IMP-004</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Deslocamento/infraestrutura</t>
+        </is>
+      </c>
+      <c r="C17" s="5" t="n">
+        <v>1300</v>
+      </c>
+      <c r="D17" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>IMP-005</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Equipamentos/materiais</t>
+        </is>
+      </c>
+      <c r="C18" s="5" t="n">
+        <v>9500</v>
+      </c>
+      <c r="D18" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>IMP-005</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Mão de obra própria</t>
+        </is>
+      </c>
+      <c r="C19" s="5" t="n">
+        <v>3500</v>
+      </c>
+      <c r="D19" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>IMP-005</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Terceiros/empreiteiros</t>
+        </is>
+      </c>
+      <c r="C20" s="5" t="n">
+        <v>3000</v>
+      </c>
+      <c r="D20" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>IMP-005</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Deslocamento/infraestrutura</t>
+        </is>
+      </c>
+      <c r="C21" s="5" t="n">
+        <v>800</v>
+      </c>
+      <c r="D21" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>IMP-006</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Equipamentos/materiais</t>
+        </is>
+      </c>
+      <c r="C22" s="5" t="n">
+        <v>29300</v>
+      </c>
+      <c r="D22" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>IMP-006</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Mão de obra própria</t>
+        </is>
+      </c>
+      <c r="C23" s="5" t="n">
+        <v>11000</v>
+      </c>
+      <c r="D23" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>IMP-006</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Terceiros/empreiteiros</t>
+        </is>
+      </c>
+      <c r="C24" s="5" t="n">
+        <v>9400</v>
+      </c>
+      <c r="D24" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>IMP-006</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Deslocamento/infraestrutura</t>
+        </is>
+      </c>
+      <c r="C25" s="5" t="n">
+        <v>2600</v>
+      </c>
+      <c r="D25" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>IMP-007</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Equipamentos/materiais</t>
+        </is>
+      </c>
+      <c r="C26" s="5" t="n">
+        <v>19900</v>
+      </c>
+      <c r="D26" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>IMP-007</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Mão de obra própria</t>
+        </is>
+      </c>
+      <c r="C27" s="5" t="n">
+        <v>7500</v>
+      </c>
+      <c r="D27" t="inlineStr"/>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>IMP-007</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Terceiros/empreiteiros</t>
+        </is>
+      </c>
+      <c r="C28" s="5" t="n">
+        <v>6400</v>
+      </c>
+      <c r="D28" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>IMP-007</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Deslocamento/infraestrutura</t>
+        </is>
+      </c>
+      <c r="C29" s="5" t="n">
+        <v>1800</v>
+      </c>
+      <c r="D29" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>IMP-008</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Equipamentos/materiais</t>
+        </is>
+      </c>
+      <c r="C30" s="5" t="n">
+        <v>11100</v>
+      </c>
+      <c r="D30" t="inlineStr"/>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>IMP-008</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Mão de obra própria</t>
+        </is>
+      </c>
+      <c r="C31" s="5" t="n">
+        <v>4200</v>
+      </c>
+      <c r="D31" t="inlineStr"/>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>IMP-008</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Terceiros/empreiteiros</t>
+        </is>
+      </c>
+      <c r="C32" s="5" t="n">
+        <v>3600</v>
+      </c>
+      <c r="D32" t="inlineStr"/>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>IMP-008</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Deslocamento/infraestrutura</t>
+        </is>
+      </c>
+      <c r="C33" s="5" t="n">
+        <v>1000</v>
+      </c>
+      <c r="D33" t="inlineStr"/>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>IMP-009</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Equipamentos/materiais</t>
+        </is>
+      </c>
+      <c r="C34" s="5" t="n">
+        <v>23100</v>
+      </c>
+      <c r="D34" t="inlineStr"/>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>IMP-009</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>Mão de obra própria</t>
+        </is>
+      </c>
+      <c r="C35" s="5" t="n">
+        <v>8700</v>
+      </c>
+      <c r="D35" t="inlineStr"/>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>IMP-009</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Terceiros/empreiteiros</t>
+        </is>
+      </c>
+      <c r="C36" s="5" t="n">
+        <v>7400</v>
+      </c>
+      <c r="D36" t="inlineStr"/>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>IMP-009</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Deslocamento/infraestrutura</t>
+        </is>
+      </c>
+      <c r="C37" s="5" t="n">
+        <v>2100</v>
+      </c>
+      <c r="D37" t="inlineStr"/>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>IMP-010</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>Equipamentos/materiais</t>
+        </is>
+      </c>
+      <c r="C38" s="5" t="n">
+        <v>10400</v>
+      </c>
+      <c r="D38" t="inlineStr"/>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>IMP-010</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>Mão de obra própria</t>
+        </is>
+      </c>
+      <c r="C39" s="5" t="n">
+        <v>3900</v>
+      </c>
+      <c r="D39" t="inlineStr"/>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>IMP-010</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Terceiros/empreiteiros</t>
+        </is>
+      </c>
+      <c r="C40" s="5" t="n">
+        <v>3300</v>
+      </c>
+      <c r="D40" t="inlineStr"/>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>IMP-010</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Deslocamento/infraestrutura</t>
+        </is>
+      </c>
+      <c r="C41" s="5" t="n">
+        <v>900</v>
+      </c>
+      <c r="D41" t="inlineStr"/>
+    </row>
+    <row r="42">
+      <c r="C42" s="5" t="n"/>
+    </row>
+    <row r="43">
+      <c r="C43" s="5" t="n"/>
+    </row>
+    <row r="44">
+      <c r="C44" s="5" t="n"/>
+    </row>
+    <row r="45">
+      <c r="C45" s="5" t="n"/>
+    </row>
+    <row r="46">
+      <c r="C46" s="5" t="n"/>
+    </row>
+    <row r="47">
+      <c r="C47" s="5" t="n"/>
+    </row>
+    <row r="48">
+      <c r="C48" s="5" t="n"/>
+    </row>
+    <row r="49">
+      <c r="C49" s="5" t="n"/>
+    </row>
+    <row r="50">
+      <c r="C50" s="5" t="n"/>
+    </row>
+    <row r="51">
+      <c r="C51" s="5" t="n"/>
+    </row>
+    <row r="52">
+      <c r="C52" s="5" t="n"/>
+    </row>
+    <row r="53">
+      <c r="C53" s="5" t="n"/>
+    </row>
+    <row r="54">
+      <c r="C54" s="5" t="n"/>
+    </row>
+    <row r="55">
+      <c r="C55" s="5" t="n"/>
+    </row>
+    <row r="56">
+      <c r="C56" s="5" t="n"/>
+    </row>
+    <row r="57">
+      <c r="C57" s="5" t="n"/>
+    </row>
+    <row r="58">
+      <c r="C58" s="5" t="n"/>
+    </row>
+    <row r="59">
+      <c r="C59" s="5" t="n"/>
+    </row>
+    <row r="60">
+      <c r="C60" s="5" t="n"/>
+    </row>
+    <row r="61">
+      <c r="C61" s="5" t="n"/>
+    </row>
+    <row r="62">
+      <c r="C62" s="5" t="n"/>
+    </row>
+    <row r="63">
+      <c r="C63" s="5" t="n"/>
+    </row>
+    <row r="64">
+      <c r="C64" s="5" t="n"/>
+    </row>
+    <row r="65">
+      <c r="C65" s="5" t="n"/>
+    </row>
+    <row r="66">
+      <c r="C66" s="5" t="n"/>
+    </row>
+    <row r="67">
+      <c r="C67" s="5" t="n"/>
+    </row>
+    <row r="68">
+      <c r="C68" s="5" t="n"/>
+    </row>
+    <row r="69">
+      <c r="C69" s="5" t="n"/>
+    </row>
+    <row r="70">
+      <c r="C70" s="5" t="n"/>
+    </row>
+    <row r="71">
+      <c r="C71" s="5" t="n"/>
+    </row>
+    <row r="72">
+      <c r="C72" s="5" t="n"/>
+    </row>
+    <row r="73">
+      <c r="C73" s="5" t="n"/>
+    </row>
+    <row r="74">
+      <c r="C74" s="5" t="n"/>
+    </row>
+    <row r="75">
+      <c r="C75" s="5" t="n"/>
+    </row>
+    <row r="76">
+      <c r="C76" s="5" t="n"/>
+    </row>
+    <row r="77">
+      <c r="C77" s="5" t="n"/>
+    </row>
+    <row r="78">
+      <c r="C78" s="5" t="n"/>
+    </row>
+    <row r="79">
+      <c r="C79" s="5" t="n"/>
+    </row>
+    <row r="80">
+      <c r="C80" s="5" t="n"/>
+    </row>
+    <row r="81">
+      <c r="C81" s="5" t="n"/>
+    </row>
+    <row r="82">
+      <c r="C82" s="5" t="n"/>
+    </row>
+    <row r="83">
+      <c r="C83" s="5" t="n"/>
+    </row>
+    <row r="84">
+      <c r="C84" s="5" t="n"/>
+    </row>
+    <row r="85">
+      <c r="C85" s="5" t="n"/>
+    </row>
+    <row r="86">
+      <c r="C86" s="5" t="n"/>
+    </row>
+    <row r="87">
+      <c r="C87" s="5" t="n"/>
+    </row>
+    <row r="88">
+      <c r="C88" s="5" t="n"/>
+    </row>
+    <row r="89">
+      <c r="C89" s="5" t="n"/>
+    </row>
+    <row r="90">
+      <c r="C90" s="5" t="n"/>
+    </row>
+    <row r="91">
+      <c r="C91" s="5" t="n"/>
+    </row>
+    <row r="92">
+      <c r="C92" s="5" t="n"/>
+    </row>
+    <row r="93">
+      <c r="C93" s="5" t="n"/>
+    </row>
+    <row r="94">
+      <c r="C94" s="5" t="n"/>
+    </row>
+    <row r="95">
+      <c r="C95" s="5" t="n"/>
+    </row>
+    <row r="96">
+      <c r="C96" s="5" t="n"/>
+    </row>
+    <row r="97">
+      <c r="C97" s="5" t="n"/>
+    </row>
+    <row r="98">
+      <c r="C98" s="5" t="n"/>
+    </row>
+    <row r="99">
+      <c r="C99" s="5" t="n"/>
+    </row>
+    <row r="100">
+      <c r="C100" s="5" t="n"/>
+    </row>
+    <row r="101">
+      <c r="C101" s="5" t="n"/>
+    </row>
+    <row r="102">
+      <c r="C102" s="5" t="n"/>
+    </row>
+    <row r="103">
+      <c r="C103" s="5" t="n"/>
+    </row>
+    <row r="104">
+      <c r="C104" s="5" t="n"/>
+    </row>
+    <row r="105">
+      <c r="C105" s="5" t="n"/>
+    </row>
+    <row r="106">
+      <c r="C106" s="5" t="n"/>
+    </row>
+    <row r="107">
+      <c r="C107" s="5" t="n"/>
+    </row>
+    <row r="108">
+      <c r="C108" s="5" t="n"/>
+    </row>
+    <row r="109">
+      <c r="C109" s="5" t="n"/>
+    </row>
+    <row r="110">
+      <c r="C110" s="5" t="n"/>
+    </row>
+    <row r="111">
+      <c r="C111" s="5" t="n"/>
+    </row>
+    <row r="112">
+      <c r="C112" s="5" t="n"/>
+    </row>
+    <row r="113">
+      <c r="C113" s="5" t="n"/>
+    </row>
+    <row r="114">
+      <c r="C114" s="5" t="n"/>
+    </row>
+    <row r="115">
+      <c r="C115" s="5" t="n"/>
+    </row>
+    <row r="116">
+      <c r="C116" s="5" t="n"/>
+    </row>
+    <row r="117">
+      <c r="C117" s="5" t="n"/>
+    </row>
+    <row r="118">
+      <c r="C118" s="5" t="n"/>
+    </row>
+    <row r="119">
+      <c r="C119" s="5" t="n"/>
+    </row>
+    <row r="120">
+      <c r="C120" s="5" t="n"/>
+    </row>
+    <row r="121">
+      <c r="C121" s="5" t="n"/>
+    </row>
+    <row r="122">
+      <c r="C122" s="5" t="n"/>
+    </row>
+    <row r="123">
+      <c r="C123" s="5" t="n"/>
+    </row>
+    <row r="124">
+      <c r="C124" s="5" t="n"/>
+    </row>
+    <row r="125">
+      <c r="C125" s="5" t="n"/>
+    </row>
+    <row r="126">
+      <c r="C126" s="5" t="n"/>
+    </row>
+    <row r="127">
+      <c r="C127" s="5" t="n"/>
+    </row>
+    <row r="128">
+      <c r="C128" s="5" t="n"/>
+    </row>
+    <row r="129">
+      <c r="C129" s="5" t="n"/>
+    </row>
+    <row r="130">
+      <c r="C130" s="5" t="n"/>
+    </row>
+    <row r="131">
+      <c r="C131" s="5" t="n"/>
+    </row>
+    <row r="132">
+      <c r="C132" s="5" t="n"/>
+    </row>
+    <row r="133">
+      <c r="C133" s="5" t="n"/>
+    </row>
+    <row r="134">
+      <c r="C134" s="5" t="n"/>
+    </row>
+    <row r="135">
+      <c r="C135" s="5" t="n"/>
+    </row>
+    <row r="136">
+      <c r="C136" s="5" t="n"/>
+    </row>
+    <row r="137">
+      <c r="C137" s="5" t="n"/>
+    </row>
+    <row r="138">
+      <c r="C138" s="5" t="n"/>
+    </row>
+    <row r="139">
+      <c r="C139" s="5" t="n"/>
+    </row>
+    <row r="140">
+      <c r="C140" s="5" t="n"/>
+    </row>
+    <row r="141">
+      <c r="C141" s="5" t="n"/>
+    </row>
+    <row r="142">
+      <c r="C142" s="5" t="n"/>
+    </row>
+    <row r="143">
+      <c r="C143" s="5" t="n"/>
+    </row>
+    <row r="144">
+      <c r="C144" s="5" t="n"/>
+    </row>
+    <row r="145">
+      <c r="C145" s="5" t="n"/>
+    </row>
+    <row r="146">
+      <c r="C146" s="5" t="n"/>
+    </row>
+    <row r="147">
+      <c r="C147" s="5" t="n"/>
+    </row>
+    <row r="148">
+      <c r="C148" s="5" t="n"/>
+    </row>
+    <row r="149">
+      <c r="C149" s="5" t="n"/>
+    </row>
+    <row r="150">
+      <c r="C150" s="5" t="n"/>
+    </row>
+    <row r="151">
+      <c r="C151" s="5" t="n"/>
+    </row>
+    <row r="152">
+      <c r="C152" s="5" t="n"/>
+    </row>
+    <row r="153">
+      <c r="C153" s="5" t="n"/>
+    </row>
+    <row r="154">
+      <c r="C154" s="5" t="n"/>
+    </row>
+    <row r="155">
+      <c r="C155" s="5" t="n"/>
+    </row>
+    <row r="156">
+      <c r="C156" s="5" t="n"/>
+    </row>
+    <row r="157">
+      <c r="C157" s="5" t="n"/>
+    </row>
+    <row r="158">
+      <c r="C158" s="5" t="n"/>
+    </row>
+    <row r="159">
+      <c r="C159" s="5" t="n"/>
+    </row>
+    <row r="160">
+      <c r="C160" s="5" t="n"/>
+    </row>
+    <row r="161">
+      <c r="C161" s="5" t="n"/>
+    </row>
+    <row r="162">
+      <c r="C162" s="5" t="n"/>
+    </row>
+    <row r="163">
+      <c r="C163" s="5" t="n"/>
+    </row>
+    <row r="164">
+      <c r="C164" s="5" t="n"/>
+    </row>
+    <row r="165">
+      <c r="C165" s="5" t="n"/>
+    </row>
+    <row r="166">
+      <c r="C166" s="5" t="n"/>
+    </row>
+    <row r="167">
+      <c r="C167" s="5" t="n"/>
+    </row>
+    <row r="168">
+      <c r="C168" s="5" t="n"/>
+    </row>
+    <row r="169">
+      <c r="C169" s="5" t="n"/>
+    </row>
+    <row r="170">
+      <c r="C170" s="5" t="n"/>
+    </row>
+    <row r="171">
+      <c r="C171" s="5" t="n"/>
+    </row>
+    <row r="172">
+      <c r="C172" s="5" t="n"/>
+    </row>
+    <row r="173">
+      <c r="C173" s="5" t="n"/>
+    </row>
+    <row r="174">
+      <c r="C174" s="5" t="n"/>
+    </row>
+    <row r="175">
+      <c r="C175" s="5" t="n"/>
+    </row>
+    <row r="176">
+      <c r="C176" s="5" t="n"/>
+    </row>
+    <row r="177">
+      <c r="C177" s="5" t="n"/>
+    </row>
+    <row r="178">
+      <c r="C178" s="5" t="n"/>
+    </row>
+    <row r="179">
+      <c r="C179" s="5" t="n"/>
+    </row>
+    <row r="180">
+      <c r="C180" s="5" t="n"/>
+    </row>
+    <row r="181">
+      <c r="C181" s="5" t="n"/>
+    </row>
+    <row r="182">
+      <c r="C182" s="5" t="n"/>
+    </row>
+    <row r="183">
+      <c r="C183" s="5" t="n"/>
+    </row>
+    <row r="184">
+      <c r="C184" s="5" t="n"/>
+    </row>
+    <row r="185">
+      <c r="C185" s="5" t="n"/>
+    </row>
+    <row r="186">
+      <c r="C186" s="5" t="n"/>
+    </row>
+    <row r="187">
+      <c r="C187" s="5" t="n"/>
+    </row>
+    <row r="188">
+      <c r="C188" s="5" t="n"/>
+    </row>
+    <row r="189">
+      <c r="C189" s="5" t="n"/>
+    </row>
+    <row r="190">
+      <c r="C190" s="5" t="n"/>
+    </row>
+    <row r="191">
+      <c r="C191" s="5" t="n"/>
+    </row>
+    <row r="192">
+      <c r="C192" s="5" t="n"/>
+    </row>
+    <row r="193">
+      <c r="C193" s="5" t="n"/>
+    </row>
+    <row r="194">
+      <c r="C194" s="5" t="n"/>
+    </row>
+    <row r="195">
+      <c r="C195" s="5" t="n"/>
+    </row>
+    <row r="196">
+      <c r="C196" s="5" t="n"/>
+    </row>
+    <row r="197">
+      <c r="C197" s="5" t="n"/>
+    </row>
+    <row r="198">
+      <c r="C198" s="5" t="n"/>
+    </row>
+    <row r="199">
+      <c r="C199" s="5" t="n"/>
+    </row>
+    <row r="200">
+      <c r="C200" s="5" t="n"/>
+    </row>
+    <row r="201">
+      <c r="C201" s="5" t="n"/>
+    </row>
+    <row r="202">
+      <c r="C202" s="5" t="n"/>
+    </row>
+    <row r="203">
+      <c r="C203" s="5" t="n"/>
+    </row>
+    <row r="204">
+      <c r="C204" s="5" t="n"/>
+    </row>
+    <row r="205">
+      <c r="C205" s="5" t="n"/>
+    </row>
+    <row r="206">
+      <c r="C206" s="5" t="n"/>
+    </row>
+    <row r="207">
+      <c r="C207" s="5" t="n"/>
+    </row>
+    <row r="208">
+      <c r="C208" s="5" t="n"/>
+    </row>
+    <row r="209">
+      <c r="C209" s="5" t="n"/>
+    </row>
+    <row r="210">
+      <c r="C210" s="5" t="n"/>
+    </row>
+    <row r="211">
+      <c r="C211" s="5" t="n"/>
+    </row>
+    <row r="212">
+      <c r="C212" s="5" t="n"/>
+    </row>
+    <row r="213">
+      <c r="C213" s="5" t="n"/>
+    </row>
+    <row r="214">
+      <c r="C214" s="5" t="n"/>
+    </row>
+    <row r="215">
+      <c r="C215" s="5" t="n"/>
+    </row>
+    <row r="216">
+      <c r="C216" s="5" t="n"/>
+    </row>
+    <row r="217">
+      <c r="C217" s="5" t="n"/>
+    </row>
+    <row r="218">
+      <c r="C218" s="5" t="n"/>
+    </row>
+    <row r="219">
+      <c r="C219" s="5" t="n"/>
+    </row>
+    <row r="220">
+      <c r="C220" s="5" t="n"/>
+    </row>
+    <row r="221">
+      <c r="C221" s="5" t="n"/>
+    </row>
+    <row r="222">
+      <c r="C222" s="5" t="n"/>
+    </row>
+    <row r="223">
+      <c r="C223" s="5" t="n"/>
+    </row>
+    <row r="224">
+      <c r="C224" s="5" t="n"/>
+    </row>
+    <row r="225">
+      <c r="C225" s="5" t="n"/>
+    </row>
+    <row r="226">
+      <c r="C226" s="5" t="n"/>
+    </row>
+    <row r="227">
+      <c r="C227" s="5" t="n"/>
+    </row>
+    <row r="228">
+      <c r="C228" s="5" t="n"/>
+    </row>
+    <row r="229">
+      <c r="C229" s="5" t="n"/>
+    </row>
+    <row r="230">
+      <c r="C230" s="5" t="n"/>
+    </row>
+    <row r="231">
+      <c r="C231" s="5" t="n"/>
+    </row>
+    <row r="232">
+      <c r="C232" s="5" t="n"/>
+    </row>
+    <row r="233">
+      <c r="C233" s="5" t="n"/>
+    </row>
+    <row r="234">
+      <c r="C234" s="5" t="n"/>
+    </row>
+    <row r="235">
+      <c r="C235" s="5" t="n"/>
+    </row>
+    <row r="236">
+      <c r="C236" s="5" t="n"/>
+    </row>
+    <row r="237">
+      <c r="C237" s="5" t="n"/>
+    </row>
+    <row r="238">
+      <c r="C238" s="5" t="n"/>
+    </row>
+    <row r="239">
+      <c r="C239" s="5" t="n"/>
+    </row>
+    <row r="240">
+      <c r="C240" s="5" t="n"/>
+    </row>
+    <row r="241">
+      <c r="C241" s="5" t="n"/>
+    </row>
+    <row r="242">
+      <c r="C242" s="5" t="n"/>
+    </row>
+    <row r="243">
+      <c r="C243" s="5" t="n"/>
+    </row>
+    <row r="244">
+      <c r="C244" s="5" t="n"/>
+    </row>
+    <row r="245">
+      <c r="C245" s="5" t="n"/>
+    </row>
+    <row r="246">
+      <c r="C246" s="5" t="n"/>
+    </row>
+    <row r="247">
+      <c r="C247" s="5" t="n"/>
+    </row>
+    <row r="248">
+      <c r="C248" s="5" t="n"/>
+    </row>
+    <row r="249">
+      <c r="C249" s="5" t="n"/>
+    </row>
+    <row r="250">
+      <c r="C250" s="5" t="n"/>
+    </row>
+    <row r="251">
+      <c r="C251" s="5" t="n"/>
+    </row>
+    <row r="252">
+      <c r="C252" s="5" t="n"/>
+    </row>
+    <row r="253">
+      <c r="C253" s="5" t="n"/>
+    </row>
+    <row r="254">
+      <c r="C254" s="5" t="n"/>
+    </row>
+    <row r="255">
+      <c r="C255" s="5" t="n"/>
+    </row>
+    <row r="256">
+      <c r="C256" s="5" t="n"/>
+    </row>
+    <row r="257">
+      <c r="C257" s="5" t="n"/>
+    </row>
+    <row r="258">
+      <c r="C258" s="5" t="n"/>
+    </row>
+    <row r="259">
+      <c r="C259" s="5" t="n"/>
+    </row>
+    <row r="260">
+      <c r="C260" s="5" t="n"/>
+    </row>
+    <row r="261">
+      <c r="C261" s="5" t="n"/>
+    </row>
+    <row r="262">
+      <c r="C262" s="5" t="n"/>
+    </row>
+    <row r="263">
+      <c r="C263" s="5" t="n"/>
+    </row>
+    <row r="264">
+      <c r="C264" s="5" t="n"/>
+    </row>
+    <row r="265">
+      <c r="C265" s="5" t="n"/>
+    </row>
+    <row r="266">
+      <c r="C266" s="5" t="n"/>
+    </row>
+    <row r="267">
+      <c r="C267" s="5" t="n"/>
+    </row>
+    <row r="268">
+      <c r="C268" s="5" t="n"/>
+    </row>
+    <row r="269">
+      <c r="C269" s="5" t="n"/>
+    </row>
+    <row r="270">
+      <c r="C270" s="5" t="n"/>
+    </row>
+    <row r="271">
+      <c r="C271" s="5" t="n"/>
+    </row>
+    <row r="272">
+      <c r="C272" s="5" t="n"/>
+    </row>
+    <row r="273">
+      <c r="C273" s="5" t="n"/>
+    </row>
+    <row r="274">
+      <c r="C274" s="5" t="n"/>
+    </row>
+    <row r="275">
+      <c r="C275" s="5" t="n"/>
+    </row>
+    <row r="276">
+      <c r="C276" s="5" t="n"/>
+    </row>
+    <row r="277">
+      <c r="C277" s="5" t="n"/>
+    </row>
+    <row r="278">
+      <c r="C278" s="5" t="n"/>
+    </row>
+    <row r="279">
+      <c r="C279" s="5" t="n"/>
+    </row>
+    <row r="280">
+      <c r="C280" s="5" t="n"/>
+    </row>
+    <row r="281">
+      <c r="C281" s="5" t="n"/>
+    </row>
+    <row r="282">
+      <c r="C282" s="5" t="n"/>
+    </row>
+    <row r="283">
+      <c r="C283" s="5" t="n"/>
+    </row>
+    <row r="284">
+      <c r="C284" s="5" t="n"/>
+    </row>
+    <row r="285">
+      <c r="C285" s="5" t="n"/>
+    </row>
+    <row r="286">
+      <c r="C286" s="5" t="n"/>
+    </row>
+    <row r="287">
+      <c r="C287" s="5" t="n"/>
+    </row>
+    <row r="288">
+      <c r="C288" s="5" t="n"/>
+    </row>
+    <row r="289">
+      <c r="C289" s="5" t="n"/>
+    </row>
+    <row r="290">
+      <c r="C290" s="5" t="n"/>
+    </row>
+    <row r="291">
+      <c r="C291" s="5" t="n"/>
+    </row>
+    <row r="292">
+      <c r="C292" s="5" t="n"/>
+    </row>
+    <row r="293">
+      <c r="C293" s="5" t="n"/>
+    </row>
+    <row r="294">
+      <c r="C294" s="5" t="n"/>
+    </row>
+    <row r="295">
+      <c r="C295" s="5" t="n"/>
+    </row>
+    <row r="296">
+      <c r="C296" s="5" t="n"/>
+    </row>
+    <row r="297">
+      <c r="C297" s="5" t="n"/>
+    </row>
+    <row r="298">
+      <c r="C298" s="5" t="n"/>
+    </row>
+    <row r="299">
+      <c r="C299" s="5" t="n"/>
+    </row>
+    <row r="300">
+      <c r="C300" s="5" t="n"/>
+    </row>
+    <row r="301">
+      <c r="C301" s="5" t="n"/>
+    </row>
+    <row r="302">
+      <c r="C302" s="5" t="n"/>
+    </row>
+    <row r="303">
+      <c r="C303" s="5" t="n"/>
+    </row>
+    <row r="304">
+      <c r="C304" s="5" t="n"/>
+    </row>
+    <row r="305">
+      <c r="C305" s="5" t="n"/>
+    </row>
+    <row r="306">
+      <c r="C306" s="5" t="n"/>
+    </row>
+    <row r="307">
+      <c r="C307" s="5" t="n"/>
+    </row>
+    <row r="308">
+      <c r="C308" s="5" t="n"/>
+    </row>
+    <row r="309">
+      <c r="C309" s="5" t="n"/>
+    </row>
+    <row r="310">
+      <c r="C310" s="5" t="n"/>
+    </row>
+    <row r="311">
+      <c r="C311" s="5" t="n"/>
+    </row>
+    <row r="312">
+      <c r="C312" s="5" t="n"/>
+    </row>
+    <row r="313">
+      <c r="C313" s="5" t="n"/>
+    </row>
+    <row r="314">
+      <c r="C314" s="5" t="n"/>
+    </row>
+    <row r="315">
+      <c r="C315" s="5" t="n"/>
+    </row>
+    <row r="316">
+      <c r="C316" s="5" t="n"/>
+    </row>
+    <row r="317">
+      <c r="C317" s="5" t="n"/>
+    </row>
+    <row r="318">
+      <c r="C318" s="5" t="n"/>
+    </row>
+    <row r="319">
+      <c r="C319" s="5" t="n"/>
+    </row>
+    <row r="320">
+      <c r="C320" s="5" t="n"/>
+    </row>
+    <row r="321">
+      <c r="C321" s="5" t="n"/>
+    </row>
+    <row r="322">
+      <c r="C322" s="5" t="n"/>
+    </row>
+    <row r="323">
+      <c r="C323" s="5" t="n"/>
+    </row>
+    <row r="324">
+      <c r="C324" s="5" t="n"/>
+    </row>
+    <row r="325">
+      <c r="C325" s="5" t="n"/>
+    </row>
+    <row r="326">
+      <c r="C326" s="5" t="n"/>
+    </row>
+    <row r="327">
+      <c r="C327" s="5" t="n"/>
+    </row>
+    <row r="328">
+      <c r="C328" s="5" t="n"/>
+    </row>
+    <row r="329">
+      <c r="C329" s="5" t="n"/>
+    </row>
+    <row r="330">
+      <c r="C330" s="5" t="n"/>
+    </row>
+    <row r="331">
+      <c r="C331" s="5" t="n"/>
+    </row>
+    <row r="332">
+      <c r="C332" s="5" t="n"/>
+    </row>
+    <row r="333">
+      <c r="C333" s="5" t="n"/>
+    </row>
+    <row r="334">
+      <c r="C334" s="5" t="n"/>
+    </row>
+    <row r="335">
+      <c r="C335" s="5" t="n"/>
+    </row>
+    <row r="336">
+      <c r="C336" s="5" t="n"/>
+    </row>
+    <row r="337">
+      <c r="C337" s="5" t="n"/>
+    </row>
+    <row r="338">
+      <c r="C338" s="5" t="n"/>
+    </row>
+    <row r="339">
+      <c r="C339" s="5" t="n"/>
+    </row>
+    <row r="340">
+      <c r="C340" s="5" t="n"/>
+    </row>
+    <row r="341">
+      <c r="C341" s="5" t="n"/>
+    </row>
+    <row r="342">
+      <c r="C342" s="5" t="n"/>
+    </row>
+    <row r="343">
+      <c r="C343" s="5" t="n"/>
+    </row>
+    <row r="344">
+      <c r="C344" s="5" t="n"/>
+    </row>
+    <row r="345">
+      <c r="C345" s="5" t="n"/>
+    </row>
+    <row r="346">
+      <c r="C346" s="5" t="n"/>
+    </row>
+    <row r="347">
+      <c r="C347" s="5" t="n"/>
+    </row>
+    <row r="348">
+      <c r="C348" s="5" t="n"/>
+    </row>
+    <row r="349">
+      <c r="C349" s="5" t="n"/>
+    </row>
+    <row r="350">
+      <c r="C350" s="5" t="n"/>
+    </row>
+    <row r="351">
+      <c r="C351" s="5" t="n"/>
+    </row>
+    <row r="352">
+      <c r="C352" s="5" t="n"/>
+    </row>
+    <row r="353">
+      <c r="C353" s="5" t="n"/>
+    </row>
+    <row r="354">
+      <c r="C354" s="5" t="n"/>
+    </row>
+    <row r="355">
+      <c r="C355" s="5" t="n"/>
+    </row>
+    <row r="356">
+      <c r="C356" s="5" t="n"/>
+    </row>
+    <row r="357">
+      <c r="C357" s="5" t="n"/>
+    </row>
+    <row r="358">
+      <c r="C358" s="5" t="n"/>
+    </row>
+    <row r="359">
+      <c r="C359" s="5" t="n"/>
+    </row>
+    <row r="360">
+      <c r="C360" s="5" t="n"/>
+    </row>
+    <row r="361">
+      <c r="C361" s="5" t="n"/>
+    </row>
+    <row r="362">
+      <c r="C362" s="5" t="n"/>
+    </row>
+    <row r="363">
+      <c r="C363" s="5" t="n"/>
+    </row>
+    <row r="364">
+      <c r="C364" s="5" t="n"/>
+    </row>
+    <row r="365">
+      <c r="C365" s="5" t="n"/>
+    </row>
+    <row r="366">
+      <c r="C366" s="5" t="n"/>
+    </row>
+    <row r="367">
+      <c r="C367" s="5" t="n"/>
+    </row>
+    <row r="368">
+      <c r="C368" s="5" t="n"/>
+    </row>
+    <row r="369">
+      <c r="C369" s="5" t="n"/>
+    </row>
+    <row r="370">
+      <c r="C370" s="5" t="n"/>
+    </row>
+    <row r="371">
+      <c r="C371" s="5" t="n"/>
+    </row>
+    <row r="372">
+      <c r="C372" s="5" t="n"/>
+    </row>
+    <row r="373">
+      <c r="C373" s="5" t="n"/>
+    </row>
+    <row r="374">
+      <c r="C374" s="5" t="n"/>
+    </row>
+    <row r="375">
+      <c r="C375" s="5" t="n"/>
+    </row>
+    <row r="376">
+      <c r="C376" s="5" t="n"/>
+    </row>
+    <row r="377">
+      <c r="C377" s="5" t="n"/>
+    </row>
+    <row r="378">
+      <c r="C378" s="5" t="n"/>
+    </row>
+    <row r="379">
+      <c r="C379" s="5" t="n"/>
+    </row>
+    <row r="380">
+      <c r="C380" s="5" t="n"/>
+    </row>
+    <row r="381">
+      <c r="C381" s="5" t="n"/>
+    </row>
+    <row r="382">
+      <c r="C382" s="5" t="n"/>
+    </row>
+    <row r="383">
+      <c r="C383" s="5" t="n"/>
+    </row>
+    <row r="384">
+      <c r="C384" s="5" t="n"/>
+    </row>
+    <row r="385">
+      <c r="C385" s="5" t="n"/>
+    </row>
+    <row r="386">
+      <c r="C386" s="5" t="n"/>
+    </row>
+    <row r="387">
+      <c r="C387" s="5" t="n"/>
+    </row>
+    <row r="388">
+      <c r="C388" s="5" t="n"/>
+    </row>
+    <row r="389">
+      <c r="C389" s="5" t="n"/>
+    </row>
+    <row r="390">
+      <c r="C390" s="5" t="n"/>
+    </row>
+    <row r="391">
+      <c r="C391" s="5" t="n"/>
+    </row>
+    <row r="392">
+      <c r="C392" s="5" t="n"/>
+    </row>
+    <row r="393">
+      <c r="C393" s="5" t="n"/>
+    </row>
+    <row r="394">
+      <c r="C394" s="5" t="n"/>
+    </row>
+    <row r="395">
+      <c r="C395" s="5" t="n"/>
+    </row>
+    <row r="396">
+      <c r="C396" s="5" t="n"/>
+    </row>
+    <row r="397">
+      <c r="C397" s="5" t="n"/>
+    </row>
+    <row r="398">
+      <c r="C398" s="5" t="n"/>
+    </row>
+    <row r="399">
+      <c r="C399" s="5" t="n"/>
+    </row>
+    <row r="400">
+      <c r="C400" s="5" t="n"/>
+    </row>
+    <row r="401">
+      <c r="C401" s="5" t="n"/>
+    </row>
+    <row r="402">
+      <c r="C402" s="5" t="n"/>
+    </row>
+    <row r="403">
+      <c r="C403" s="5" t="n"/>
+    </row>
+    <row r="404">
+      <c r="C404" s="5" t="n"/>
+    </row>
+    <row r="405">
+      <c r="C405" s="5" t="n"/>
+    </row>
+    <row r="406">
+      <c r="C406" s="5" t="n"/>
+    </row>
+    <row r="407">
+      <c r="C407" s="5" t="n"/>
+    </row>
+    <row r="408">
+      <c r="C408" s="5" t="n"/>
+    </row>
+    <row r="409">
+      <c r="C409" s="5" t="n"/>
+    </row>
+    <row r="410">
+      <c r="C410" s="5" t="n"/>
+    </row>
+    <row r="411">
+      <c r="C411" s="5" t="n"/>
+    </row>
+    <row r="412">
+      <c r="C412" s="5" t="n"/>
+    </row>
+    <row r="413">
+      <c r="C413" s="5" t="n"/>
+    </row>
+    <row r="414">
+      <c r="C414" s="5" t="n"/>
+    </row>
+    <row r="415">
+      <c r="C415" s="5" t="n"/>
+    </row>
+    <row r="416">
+      <c r="C416" s="5" t="n"/>
+    </row>
+    <row r="417">
+      <c r="C417" s="5" t="n"/>
+    </row>
+    <row r="418">
+      <c r="C418" s="5" t="n"/>
+    </row>
+    <row r="419">
+      <c r="C419" s="5" t="n"/>
+    </row>
+    <row r="420">
+      <c r="C420" s="5" t="n"/>
+    </row>
+    <row r="421">
+      <c r="C421" s="5" t="n"/>
+    </row>
+    <row r="422">
+      <c r="C422" s="5" t="n"/>
+    </row>
+    <row r="423">
+      <c r="C423" s="5" t="n"/>
+    </row>
+    <row r="424">
+      <c r="C424" s="5" t="n"/>
+    </row>
+    <row r="425">
+      <c r="C425" s="5" t="n"/>
+    </row>
+    <row r="426">
+      <c r="C426" s="5" t="n"/>
+    </row>
+    <row r="427">
+      <c r="C427" s="5" t="n"/>
+    </row>
+    <row r="428">
+      <c r="C428" s="5" t="n"/>
+    </row>
+    <row r="429">
+      <c r="C429" s="5" t="n"/>
+    </row>
+    <row r="430">
+      <c r="C430" s="5" t="n"/>
+    </row>
+    <row r="431">
+      <c r="C431" s="5" t="n"/>
+    </row>
+    <row r="432">
+      <c r="C432" s="5" t="n"/>
+    </row>
+    <row r="433">
+      <c r="C433" s="5" t="n"/>
+    </row>
+    <row r="434">
+      <c r="C434" s="5" t="n"/>
+    </row>
+    <row r="435">
+      <c r="C435" s="5" t="n"/>
+    </row>
+    <row r="436">
+      <c r="C436" s="5" t="n"/>
+    </row>
+    <row r="437">
+      <c r="C437" s="5" t="n"/>
+    </row>
+    <row r="438">
+      <c r="C438" s="5" t="n"/>
+    </row>
+    <row r="439">
+      <c r="C439" s="5" t="n"/>
+    </row>
+    <row r="440">
+      <c r="C440" s="5" t="n"/>
+    </row>
+    <row r="441">
+      <c r="C441" s="5" t="n"/>
+    </row>
+    <row r="442">
+      <c r="C442" s="5" t="n"/>
+    </row>
+    <row r="443">
+      <c r="C443" s="5" t="n"/>
+    </row>
+    <row r="444">
+      <c r="C444" s="5" t="n"/>
+    </row>
+    <row r="445">
+      <c r="C445" s="5" t="n"/>
+    </row>
+    <row r="446">
+      <c r="C446" s="5" t="n"/>
+    </row>
+    <row r="447">
+      <c r="C447" s="5" t="n"/>
+    </row>
+    <row r="448">
+      <c r="C448" s="5" t="n"/>
+    </row>
+    <row r="449">
+      <c r="C449" s="5" t="n"/>
+    </row>
+    <row r="450">
+      <c r="C450" s="5" t="n"/>
+    </row>
+    <row r="451">
+      <c r="C451" s="5" t="n"/>
+    </row>
+    <row r="452">
+      <c r="C452" s="5" t="n"/>
+    </row>
+    <row r="453">
+      <c r="C453" s="5" t="n"/>
+    </row>
+    <row r="454">
+      <c r="C454" s="5" t="n"/>
+    </row>
+    <row r="455">
+      <c r="C455" s="5" t="n"/>
+    </row>
+    <row r="456">
+      <c r="C456" s="5" t="n"/>
+    </row>
+    <row r="457">
+      <c r="C457" s="5" t="n"/>
+    </row>
+    <row r="458">
+      <c r="C458" s="5" t="n"/>
+    </row>
+    <row r="459">
+      <c r="C459" s="5" t="n"/>
+    </row>
+    <row r="460">
+      <c r="C460" s="5" t="n"/>
+    </row>
+    <row r="461">
+      <c r="C461" s="5" t="n"/>
+    </row>
+    <row r="462">
+      <c r="C462" s="5" t="n"/>
+    </row>
+    <row r="463">
+      <c r="C463" s="5" t="n"/>
+    </row>
+    <row r="464">
+      <c r="C464" s="5" t="n"/>
+    </row>
+    <row r="465">
+      <c r="C465" s="5" t="n"/>
+    </row>
+    <row r="466">
+      <c r="C466" s="5" t="n"/>
+    </row>
+    <row r="467">
+      <c r="C467" s="5" t="n"/>
+    </row>
+    <row r="468">
+      <c r="C468" s="5" t="n"/>
+    </row>
+    <row r="469">
+      <c r="C469" s="5" t="n"/>
+    </row>
+    <row r="470">
+      <c r="C470" s="5" t="n"/>
+    </row>
+    <row r="471">
+      <c r="C471" s="5" t="n"/>
+    </row>
+    <row r="472">
+      <c r="C472" s="5" t="n"/>
+    </row>
+    <row r="473">
+      <c r="C473" s="5" t="n"/>
+    </row>
+    <row r="474">
+      <c r="C474" s="5" t="n"/>
+    </row>
+    <row r="475">
+      <c r="C475" s="5" t="n"/>
+    </row>
+    <row r="476">
+      <c r="C476" s="5" t="n"/>
+    </row>
+    <row r="477">
+      <c r="C477" s="5" t="n"/>
+    </row>
+    <row r="478">
+      <c r="C478" s="5" t="n"/>
+    </row>
+    <row r="479">
+      <c r="C479" s="5" t="n"/>
+    </row>
+    <row r="480">
+      <c r="C480" s="5" t="n"/>
+    </row>
+    <row r="481">
+      <c r="C481" s="5" t="n"/>
+    </row>
+    <row r="482">
+      <c r="C482" s="5" t="n"/>
+    </row>
+    <row r="483">
+      <c r="C483" s="5" t="n"/>
+    </row>
+    <row r="484">
+      <c r="C484" s="5" t="n"/>
+    </row>
+    <row r="485">
+      <c r="C485" s="5" t="n"/>
+    </row>
+    <row r="486">
+      <c r="C486" s="5" t="n"/>
+    </row>
+    <row r="487">
+      <c r="C487" s="5" t="n"/>
+    </row>
+    <row r="488">
+      <c r="C488" s="5" t="n"/>
+    </row>
+    <row r="489">
+      <c r="C489" s="5" t="n"/>
+    </row>
+    <row r="490">
+      <c r="C490" s="5" t="n"/>
+    </row>
+    <row r="491">
+      <c r="C491" s="5" t="n"/>
+    </row>
+    <row r="492">
+      <c r="C492" s="5" t="n"/>
+    </row>
+    <row r="493">
+      <c r="C493" s="5" t="n"/>
+    </row>
+    <row r="494">
+      <c r="C494" s="5" t="n"/>
+    </row>
+    <row r="495">
+      <c r="C495" s="5" t="n"/>
+    </row>
+    <row r="496">
+      <c r="C496" s="5" t="n"/>
+    </row>
+    <row r="497">
+      <c r="C497" s="5" t="n"/>
+    </row>
+    <row r="498">
+      <c r="C498" s="5" t="n"/>
+    </row>
+    <row r="499">
+      <c r="C499" s="5" t="n"/>
+    </row>
+    <row r="500">
+      <c r="C500" s="5" t="n"/>
+    </row>
+  </sheetData>
+  <dataValidations count="2">
+    <dataValidation sqref="B2:B500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="Escolha um valor da lista" type="list">
+      <formula1>"Equipamentos/materiais,Mão de obra própria,Terceiros/empreiteiros,Deslocamento/infraestrutura"</formula1>
+    </dataValidation>
+    <dataValidation sqref="A2:A500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>Implantacoes!$A$2:$A$500</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:H500"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -7078,7 +8642,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>